<commit_message>
Load the Finance Director's tuning grid into the bucket rules; re-run and re-verify all twelve months
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PdcnbvMxTN9eaMqR4tfx6H
</commit_message>
<xml_diff>
--- a/output/model_reports/Model_Report_2025_M03.xlsx
+++ b/output/model_reports/Model_Report_2025_M03.xlsx
@@ -1010,13 +1010,13 @@
         <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>6221.038</v>
+        <v>21257.21</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>6221.038</v>
+        <v>21257.21</v>
       </c>
     </row>
     <row r="3">
@@ -1032,13 +1032,13 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>317960.009</v>
+        <v>259215.555</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>185478.41</v>
+        <v>179444.201</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>503438.419</v>
+        <v>438659.756</v>
       </c>
     </row>
     <row r="4">
@@ -1054,13 +1054,13 @@
         <v>0</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>1726.948</v>
+        <v>21105.629</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0</v>
+        <v>6034.209</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1726.948</v>
+        <v>27139.838</v>
       </c>
     </row>
     <row r="5">
@@ -1120,13 +1120,13 @@
         <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>95482.465</v>
+        <v>119812.066</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>95482.465</v>
+        <v>119812.066</v>
       </c>
     </row>
     <row r="8">
@@ -1239,28 +1239,28 @@
         <v>32617.62</v>
       </c>
       <c r="C2" s="7" t="n">
-        <v>326.176</v>
+        <v>1630.881</v>
       </c>
       <c r="D2" s="7" t="n">
-        <v>30986.739</v>
+        <v>26094.096</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>1304.705</v>
+        <v>1630.881</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>0</v>
+        <v>3261.762</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.009999993868344777</v>
+        <v>0.05</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>0.95</v>
+        <v>0.7999999999999999</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>0.04000000613165522</v>
+        <v>0.05</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>0</v>
+        <v>0.09999999999999999</v>
       </c>
     </row>
     <row r="3">
@@ -1273,28 +1273,28 @@
         <v>241587.59</v>
       </c>
       <c r="C3" s="7" t="n">
-        <v>4831.752</v>
+        <v>12079.379</v>
       </c>
       <c r="D3" s="7" t="n">
-        <v>236755.838</v>
+        <v>181190.693</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0</v>
+        <v>12079.379</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>0</v>
+        <v>36238.139</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.0200000008278571</v>
+        <v>0.04999999793035727</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>0.9799999991721429</v>
+        <v>0.7500000020696428</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>0</v>
+        <v>0.04999999793035727</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>0</v>
+        <v>0.1500000020696428</v>
       </c>
     </row>
     <row r="4">
@@ -1304,31 +1304,31 @@
         </is>
       </c>
       <c r="B4" s="7" t="n">
-        <v>16447.64</v>
+        <v>16447.639</v>
       </c>
       <c r="C4" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>9116.594999999999</v>
+        <v>7293.276</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>0</v>
+        <v>911.659</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>7331.045</v>
+        <v>8242.704</v>
       </c>
       <c r="G4" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>0.5542798237315505</v>
+        <v>0.4434238859449676</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>0</v>
+        <v>0.05542795534362106</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>0.4457201762684495</v>
+        <v>0.5011481587114114</v>
       </c>
     </row>
     <row r="5">
@@ -1375,28 +1375,28 @@
         <v>88151.42</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>0</v>
+        <v>4407.571</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>0</v>
+        <v>8815.142</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>0</v>
+        <v>4407.571</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>88151.42</v>
+        <v>70521.136</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="7">
@@ -1406,31 +1406,31 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>30966.43</v>
+        <v>30966.431</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>0</v>
+        <v>1548.322</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>30966.43</v>
+        <v>26321.465</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0</v>
+        <v>1548.322</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>0</v>
+        <v>1548.322</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0</v>
+        <v>0.05000001453186517</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>1</v>
+        <v>0.8499999564044045</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>0</v>
+        <v>0.05000001453186517</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>0</v>
+        <v>0.05000001453186517</v>
       </c>
     </row>
     <row r="8">
@@ -1440,28 +1440,28 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>10556.61</v>
+        <v>10556.611</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>0</v>
+        <v>527.831</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>10134.346</v>
+        <v>9500.949000000001</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>422.264</v>
+        <v>527.831</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>0</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>0</v>
+        <v>0.05000004262731667</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>0.9600000378909518</v>
+        <v>0.8999999147453667</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>0.03999996210904827</v>
+        <v>0.05000004262731667</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>0</v>
@@ -1480,10 +1480,10 @@
         <v>0</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>120683.61</v>
+        <v>114649.429</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0</v>
+        <v>6034.181</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>0</v>
@@ -1492,10 +1492,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>1</v>
+        <v>0.9499999958569354</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>0</v>
+        <v>0.05000000414306466</v>
       </c>
       <c r="J9" s="4" t="n">
         <v>0</v>
@@ -1733,13 +1733,13 @@
         </is>
       </c>
       <c r="B2" s="7" t="n">
-        <v>6221.078</v>
+        <v>21257.134</v>
       </c>
       <c r="C2" s="7" t="n">
-        <v>326.176</v>
+        <v>1630.881</v>
       </c>
       <c r="D2" s="7" t="n">
-        <v>4831.752</v>
+        <v>12079.379</v>
       </c>
       <c r="E2" s="7" t="n">
         <v>0</v>
@@ -1748,13 +1748,13 @@
         <v>1063.15</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>0</v>
+        <v>4407.571</v>
       </c>
       <c r="H2" s="7" t="n">
-        <v>0</v>
+        <v>1548.322</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>0</v>
+        <v>527.831</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>0</v>
@@ -1766,25 +1766,25 @@
         <v>0</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>0.05243078450390751</v>
+        <v>0.07672158438668167</v>
       </c>
       <c r="N2" s="4" t="n">
-        <v>0.7766743963023772</v>
+        <v>0.568250592953876</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>0</v>
       </c>
       <c r="P2" s="4" t="n">
-        <v>0.1708948191937153</v>
+        <v>0.05001379772080281</v>
       </c>
       <c r="Q2" s="4" t="n">
-        <v>0</v>
+        <v>0.2073454963401933</v>
       </c>
       <c r="R2" s="4" t="n">
-        <v>0</v>
+        <v>0.07283775884368983</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0</v>
+        <v>0.02483076975475621</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0</v>
@@ -1803,31 +1803,31 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>503438.358</v>
+        <v>438659.85</v>
       </c>
       <c r="C3" s="7" t="n">
-        <v>30986.739</v>
+        <v>26094.096</v>
       </c>
       <c r="D3" s="7" t="n">
-        <v>236755.838</v>
+        <v>181190.693</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>9116.594999999999</v>
+        <v>7293.276</v>
       </c>
       <c r="F3" s="7" t="n">
         <v>0</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>0</v>
+        <v>8815.142</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>30966.43</v>
+        <v>26321.465</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>10134.346</v>
+        <v>9500.949000000001</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>120683.61</v>
+        <v>114649.429</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>2524.8</v>
@@ -1836,34 +1836,34 @@
         <v>62270</v>
       </c>
       <c r="M3" s="4" t="n">
-        <v>0.06155021465408482</v>
+        <v>0.05948594565926196</v>
       </c>
       <c r="N3" s="4" t="n">
-        <v>0.4702777097489262</v>
+        <v>0.413055110924786</v>
       </c>
       <c r="O3" s="4" t="n">
-        <v>0.0181086618751446</v>
+        <v>0.01662626748265199</v>
       </c>
       <c r="P3" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q3" s="4" t="n">
-        <v>0</v>
+        <v>0.02009562078681238</v>
       </c>
       <c r="R3" s="4" t="n">
-        <v>0.06150987406486019</v>
+        <v>0.06000427210286057</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.02013026190586773</v>
+        <v>0.02165903489913654</v>
       </c>
       <c r="T3" s="4" t="n">
-        <v>0.2397187422893986</v>
+        <v>0.2613629421521026</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.0050151124956593</v>
+        <v>0.005755712541277713</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.1236894229660585</v>
+        <v>0.1419550934511102</v>
       </c>
     </row>
     <row r="4">
@@ -1873,31 +1873,31 @@
         </is>
       </c>
       <c r="B4" s="7" t="n">
-        <v>1726.969</v>
+        <v>27139.824</v>
       </c>
       <c r="C4" s="7" t="n">
-        <v>1304.705</v>
+        <v>1630.881</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>0</v>
+        <v>12079.379</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>0</v>
+        <v>911.659</v>
       </c>
       <c r="F4" s="7" t="n">
         <v>0</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>0</v>
+        <v>4407.571</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>0</v>
+        <v>1548.322</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>422.264</v>
+        <v>527.831</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>0</v>
+        <v>6034.181</v>
       </c>
       <c r="K4" s="7" t="n">
         <v>0</v>
@@ -1906,28 +1906,28 @@
         <v>0</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>0.7554883729817964</v>
+        <v>0.06009180457470911</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>0</v>
+        <v>0.4450794890932233</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>0</v>
+        <v>0.03359119056925351</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>0</v>
+        <v>0.1624023427712722</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>0</v>
+        <v>0.05704981727221223</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.2445116270182036</v>
+        <v>0.01944857859063493</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>0</v>
+        <v>0.2223367771286947</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>0</v>
@@ -1943,25 +1943,25 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>95482.465</v>
+        <v>119812.063</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>0</v>
+        <v>3261.762</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>0</v>
+        <v>36238.139</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>7331.045</v>
+        <v>8242.704</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>0</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>88151.42</v>
+        <v>70521.136</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0</v>
+        <v>1548.322</v>
       </c>
       <c r="I5" s="7" t="n">
         <v>0</v>
@@ -1976,22 +1976,22 @@
         <v>0</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>0</v>
+        <v>0.02722398661977801</v>
       </c>
       <c r="N5" s="4" t="n">
-        <v>0</v>
+        <v>0.3024581840311021</v>
       </c>
       <c r="O5" s="4" t="n">
-        <v>0.07677896669299436</v>
+        <v>0.06879694576329931</v>
       </c>
       <c r="P5" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q5" s="4" t="n">
-        <v>0.9232210333070057</v>
+        <v>0.5885979611251665</v>
       </c>
       <c r="R5" s="4" t="n">
-        <v>0</v>
+        <v>0.01292292246065407</v>
       </c>
       <c r="S5" s="4" t="n">
         <v>0</v>
@@ -2086,16 +2086,16 @@
         </is>
       </c>
       <c r="B2" s="7" t="n">
-        <v>326.176</v>
+        <v>1630.881</v>
       </c>
       <c r="C2" s="7" t="n">
-        <v>30986.739</v>
+        <v>26094.096</v>
       </c>
       <c r="D2" s="7" t="n">
-        <v>1304.705</v>
+        <v>1630.881</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>0</v>
+        <v>3261.762</v>
       </c>
       <c r="F2" s="7" t="n">
         <v>32617.62</v>
@@ -2104,7 +2104,7 @@
         <v>32617.62</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>0.95</v>
+        <v>0.7999999999999999</v>
       </c>
     </row>
     <row r="3">
@@ -2114,16 +2114,16 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>4831.752</v>
+        <v>12079.379</v>
       </c>
       <c r="C3" s="7" t="n">
-        <v>236755.838</v>
+        <v>181190.693</v>
       </c>
       <c r="D3" s="7" t="n">
-        <v>0</v>
+        <v>12079.379</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0</v>
+        <v>36238.139</v>
       </c>
       <c r="F3" s="7" t="n">
         <v>241587.59</v>
@@ -2132,7 +2132,7 @@
         <v>241587.59</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>0.9799999991721429</v>
+        <v>0.7500000020696428</v>
       </c>
     </row>
     <row r="4">
@@ -2145,22 +2145,22 @@
         <v>0</v>
       </c>
       <c r="C4" s="7" t="n">
-        <v>9116.594999999999</v>
+        <v>7293.276</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>0</v>
+        <v>911.659</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>7331.045</v>
+        <v>8242.704</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>16447.64</v>
+        <v>16447.639</v>
       </c>
       <c r="G4" s="7" t="n">
         <v>16447.64</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>0.5542798237315505</v>
+        <v>0.4434238859449676</v>
       </c>
     </row>
     <row r="5">
@@ -2198,16 +2198,16 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>0</v>
+        <v>4407.571</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>0</v>
+        <v>8815.142</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>0</v>
+        <v>4407.571</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>88151.42</v>
+        <v>70521.136</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>88151.42</v>
@@ -2216,7 +2216,7 @@
         <v>88151.42</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="7">
@@ -2226,25 +2226,25 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>0</v>
+        <v>1548.322</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>30966.43</v>
+        <v>26321.465</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>0</v>
+        <v>1548.322</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0</v>
+        <v>1548.322</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>30966.43</v>
+        <v>30966.431</v>
       </c>
       <c r="G7" s="7" t="n">
         <v>30966.43</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>1</v>
+        <v>0.8499999564044045</v>
       </c>
     </row>
     <row r="8">
@@ -2254,25 +2254,25 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>0</v>
+        <v>527.831</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>10134.346</v>
+        <v>9500.949000000001</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>422.264</v>
+        <v>527.831</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>10556.61</v>
+        <v>10556.611</v>
       </c>
       <c r="G8" s="7" t="n">
         <v>10556.61</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>0.9600000378909518</v>
+        <v>0.8999999147453667</v>
       </c>
     </row>
     <row r="9">
@@ -2285,10 +2285,10 @@
         <v>0</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>120683.61</v>
+        <v>114649.429</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>0</v>
+        <v>6034.181</v>
       </c>
       <c r="E9" s="7" t="n">
         <v>0</v>
@@ -2300,7 +2300,7 @@
         <v>120683.61</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>1</v>
+        <v>0.9499999958569354</v>
       </c>
     </row>
     <row r="10">
@@ -2366,19 +2366,19 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>6221.078</v>
+        <v>21257.134</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>503438.358</v>
+        <v>438659.85</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>1726.969</v>
+        <v>27139.824</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>95482.465</v>
+        <v>119812.063</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>606868.87</v>
+        <v>606868.871</v>
       </c>
       <c r="G12" s="8" t="n">
         <v>606868.87</v>
@@ -2503,13 +2503,13 @@
         <v>5080.522</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>5339.947</v>
+        <v>5446.319</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>16026.174</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>11886.155</v>
+        <v>10487.4</v>
       </c>
       <c r="L2" t="inlineStr"/>
     </row>
@@ -2543,13 +2543,13 @@
         <v>5079.041</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>5337.87</v>
+        <v>5428.033</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>15847.883</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>11781.828</v>
+        <v>10407.989</v>
       </c>
       <c r="L3" t="inlineStr"/>
     </row>
@@ -2583,13 +2583,13 @@
         <v>5056.556</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>5306.616</v>
+        <v>5244.798</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>14402.764</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>10104.572</v>
+        <v>8994.002</v>
       </c>
       <c r="L4" t="inlineStr"/>
     </row>
@@ -2623,13 +2623,13 @@
         <v>5053.513</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>5302.386</v>
+        <v>5217.257</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>14191.015</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>9878.013000000001</v>
+        <v>8805.777</v>
       </c>
       <c r="L5" t="inlineStr"/>
     </row>
@@ -2663,13 +2663,13 @@
         <v>5026.998</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>5265.53</v>
+        <v>5000.621</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>12317.203</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>7899.999</v>
+        <v>7141.126</v>
       </c>
       <c r="L6" t="inlineStr"/>
     </row>
@@ -2703,13 +2703,13 @@
         <v>2546.455</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>2678.574</v>
+        <v>2769.414</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>8466.453</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>6408.465</v>
+        <v>5641.558</v>
       </c>
       <c r="L7" t="inlineStr"/>
     </row>
@@ -2743,13 +2743,13 @@
         <v>2546.454</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>2678.573</v>
+        <v>2769.414</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>8466.453</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>6408.466</v>
+        <v>5641.558</v>
       </c>
       <c r="L8" t="inlineStr"/>
     </row>
@@ -2783,13 +2783,13 @@
         <v>2533.021</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>2659.9</v>
+        <v>2659.3</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>7505.791</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>5406.741</v>
+        <v>4797.919</v>
       </c>
       <c r="L9" t="inlineStr"/>
     </row>
@@ -2823,13 +2823,13 @@
         <v>2532.014</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>2658.501</v>
+        <v>2647.451</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>7395.223</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>5333.226</v>
+        <v>4740.345</v>
       </c>
       <c r="L10" t="inlineStr"/>
     </row>
@@ -2863,13 +2863,13 @@
         <v>2527.368</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>2652.043</v>
+        <v>2610.929</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>7122.626</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>4986.044</v>
+        <v>4446.071</v>
       </c>
       <c r="L11" t="inlineStr"/>
     </row>
@@ -2903,13 +2903,13 @@
         <v>2525.671</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>2649.684</v>
+        <v>2598.812</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>7024.084</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>4858.997</v>
+        <v>4336.613</v>
       </c>
       <c r="L12" t="inlineStr"/>
     </row>
@@ -2943,13 +2943,13 @@
         <v>2273.678</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>2647.519</v>
+        <v>2806.983</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>7770.859</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>8668.971</v>
+        <v>7754.306</v>
       </c>
       <c r="L13" t="inlineStr"/>
     </row>
@@ -2983,13 +2983,13 @@
         <v>2046.31</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>2382.767</v>
+        <v>2526.285</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>6993.773</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>7802.073</v>
+        <v>6978.875</v>
       </c>
       <c r="L14" t="inlineStr"/>
     </row>
@@ -3023,13 +3023,13 @@
         <v>2046.31</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>2382.767</v>
+        <v>2526.285</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>6993.773</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>7802.073</v>
+        <v>6978.875</v>
       </c>
       <c r="L15" t="inlineStr"/>
     </row>
@@ -3063,13 +3063,13 @@
         <v>1922.204</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>2070.999</v>
+        <v>1920.169</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>3729.597</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>3326.537</v>
+        <v>3083.945</v>
       </c>
       <c r="L16" t="inlineStr"/>
     </row>
@@ -3103,13 +3103,13 @@
         <v>1747.538</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>1882.83</v>
+        <v>1584.895</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>1766.593</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>729.422</v>
+        <v>808.398</v>
       </c>
       <c r="L17" t="inlineStr"/>
     </row>
@@ -3143,13 +3143,13 @@
         <v>1577.92</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>1626.233</v>
+        <v>1580.352</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>4319.469</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>2958.476</v>
+        <v>2653.351</v>
       </c>
       <c r="L18" t="inlineStr"/>
     </row>
@@ -3183,13 +3183,13 @@
         <v>1411.661</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>1411.661</v>
+        <v>1129.329</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>1101.096</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>0</v>
+        <v>141.166</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -3227,13 +3227,13 @@
         <v>1364.207</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>1588.512</v>
+        <v>1684.191</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>4662.515</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>5201.382</v>
+        <v>4652.582</v>
       </c>
       <c r="L20" t="inlineStr"/>
     </row>
@@ -3267,13 +3267,13 @@
         <v>1354.732</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>1444.374</v>
+        <v>1876.596</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>7269.138</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>10897.31</v>
+        <v>9686.26</v>
       </c>
       <c r="L21" t="inlineStr"/>
     </row>
@@ -3307,13 +3307,13 @@
         <v>1328.422</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>1400.942</v>
+        <v>1227.481</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>1851.354</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>1301.745</v>
+        <v>1263.184</v>
       </c>
       <c r="L22" t="inlineStr"/>
     </row>
@@ -3347,13 +3347,13 @@
         <v>1209.995</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>1209.995</v>
+        <v>967.996</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>943.796</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>0</v>
+        <v>120.999</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -3391,13 +3391,13 @@
         <v>1209.995</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>1209.995</v>
+        <v>967.996</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>943.796</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>0</v>
+        <v>120.999</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -3435,13 +3435,13 @@
         <v>913.739</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>1064.939</v>
+        <v>1195.815</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>3400.209</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>3769.255</v>
+        <v>3311.068</v>
       </c>
       <c r="L25" t="inlineStr"/>
     </row>
@@ -3475,13 +3475,13 @@
         <v>689.848</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>805.021</v>
+        <v>926.446</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>2788.489</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>3167.589</v>
+        <v>2779.541</v>
       </c>
       <c r="L26" t="inlineStr"/>
     </row>
@@ -3515,13 +3515,13 @@
         <v>665.158</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>701.492</v>
+        <v>615.5650000000001</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>937.135</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>664.928</v>
+        <v>643.933</v>
       </c>
       <c r="L27" t="inlineStr"/>
     </row>
@@ -3555,13 +3555,13 @@
         <v>665.158</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>701.492</v>
+        <v>615.5650000000001</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>937.135</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>664.928</v>
+        <v>643.933</v>
       </c>
       <c r="L28" t="inlineStr"/>
     </row>
@@ -3595,13 +3595,13 @@
         <v>665.158</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>701.491</v>
+        <v>615.564</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>937.135</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>664.929</v>
+        <v>643.934</v>
       </c>
       <c r="L29" t="inlineStr"/>
     </row>
@@ -3635,13 +3635,13 @@
         <v>665.158</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>701.491</v>
+        <v>615.564</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>937.135</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>664.929</v>
+        <v>643.934</v>
       </c>
       <c r="L30" t="inlineStr"/>
     </row>
@@ -3675,13 +3675,13 @@
         <v>665.158</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>701.492</v>
+        <v>615.5650000000001</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>937.135</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>664.928</v>
+        <v>643.933</v>
       </c>
       <c r="L31" t="inlineStr"/>
     </row>
@@ -3715,13 +3715,13 @@
         <v>635.553</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>635.553</v>
+        <v>508.442</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>494.814</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>0</v>
+        <v>63.555</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -3759,13 +3759,13 @@
         <v>469.435</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>549.936</v>
+        <v>656.942</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>2331.379</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>2835.738</v>
+        <v>2509.4</v>
       </c>
       <c r="L33" t="inlineStr"/>
     </row>
@@ -3799,13 +3799,13 @@
         <v>469.04</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>549.386</v>
+        <v>654.3869999999999</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>2308.463</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>2806.186</v>
+        <v>2483.555</v>
       </c>
       <c r="L34" t="inlineStr"/>
     </row>
@@ -3839,13 +3839,13 @@
         <v>469.04</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>549.386</v>
+        <v>654.3869999999999</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>2308.463</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>2806.186</v>
+        <v>2483.555</v>
       </c>
       <c r="L35" t="inlineStr"/>
     </row>
@@ -3879,13 +3879,13 @@
         <v>464.693</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>543.3440000000001</v>
+        <v>626.125</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>2079.908</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>2480.3</v>
+        <v>2200.164</v>
       </c>
       <c r="L36" t="inlineStr"/>
     </row>
@@ -3919,13 +3919,13 @@
         <v>462.085</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>539.7190000000001</v>
+        <v>627.091</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>1965.631</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>2277.584</v>
+        <v>2002.814</v>
       </c>
       <c r="L37" t="inlineStr"/>
     </row>
@@ -3959,13 +3959,13 @@
         <v>462.085</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>539.7190000000001</v>
+        <v>627.091</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>1965.631</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>2277.584</v>
+        <v>2002.814</v>
       </c>
       <c r="L38" t="inlineStr"/>
     </row>
@@ -3999,13 +3999,13 @@
         <v>457.521</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>533.375</v>
+        <v>595.758</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>1760.605</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>1936.509</v>
+        <v>1707.903</v>
       </c>
       <c r="L39" t="inlineStr"/>
     </row>
@@ -4039,13 +4039,13 @@
         <v>455.525</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>530.601</v>
+        <v>596.627</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>1645.716</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>1780.856</v>
+        <v>1556.622</v>
       </c>
       <c r="L40" t="inlineStr"/>
     </row>
@@ -4079,13 +4079,13 @@
         <v>455.13</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>530.052</v>
+        <v>563.951</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>1577.088</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>1763.355</v>
+        <v>1576.702</v>
       </c>
       <c r="L41" t="inlineStr"/>
     </row>
@@ -4119,13 +4119,13 @@
         <v>454.735</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>529.503</v>
+        <v>561.395</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>1554.172</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>1733.796</v>
+        <v>1550.864</v>
       </c>
       <c r="L42" t="inlineStr"/>
     </row>
@@ -4159,13 +4159,13 @@
         <v>451.968</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>525.6559999999999</v>
+        <v>546.248</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>1454.914</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>1525.063</v>
+        <v>1365.865</v>
       </c>
       <c r="L43" t="inlineStr"/>
     </row>
@@ -4199,13 +4199,13 @@
         <v>432.447</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>498.522</v>
+        <v>416.864</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>446.525</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>62.647</v>
+        <v>97.128</v>
       </c>
       <c r="L44" t="inlineStr"/>
     </row>
@@ -4239,13 +4239,13 @@
         <v>403.332</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>403.332</v>
+        <v>322.666</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>314.599</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>0</v>
+        <v>40.332</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
@@ -4283,13 +4283,13 @@
         <v>302.499</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>302.499</v>
+        <v>241.999</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>235.949</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>0</v>
+        <v>30.25</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
@@ -4327,13 +4327,13 @@
         <v>302.499</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>302.499</v>
+        <v>241.999</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>235.949</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>0</v>
+        <v>30.25</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
@@ -4371,13 +4371,13 @@
         <v>302.499</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>302.499</v>
+        <v>241.999</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>235.949</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>0</v>
+        <v>30.25</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
@@ -4415,13 +4415,13 @@
         <v>302.499</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>302.499</v>
+        <v>241.999</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>235.949</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>0</v>
+        <v>30.25</v>
       </c>
       <c r="L49" t="inlineStr">
         <is>
@@ -4459,13 +4459,13 @@
         <v>302.499</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>302.499</v>
+        <v>241.999</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>235.949</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>0</v>
+        <v>30.25</v>
       </c>
       <c r="L50" t="inlineStr">
         <is>
@@ -4503,13 +4503,13 @@
         <v>302.499</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>302.499</v>
+        <v>241.999</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>235.949</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>0</v>
+        <v>30.25</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
@@ -4547,13 +4547,13 @@
         <v>236.63</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>277.626</v>
+        <v>345.608</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>1291.395</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>1559.691</v>
+        <v>1372.202</v>
       </c>
       <c r="L52" t="inlineStr"/>
     </row>
@@ -4587,13 +4587,13 @@
         <v>234.717</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>274.968</v>
+        <v>328.471</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>1417.871</v>
+        <v>1254.701</v>
       </c>
       <c r="L53" t="inlineStr"/>
     </row>
@@ -4627,13 +4627,13 @@
         <v>234.717</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>274.968</v>
+        <v>328.471</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>1417.871</v>
+        <v>1254.701</v>
       </c>
       <c r="L54" t="inlineStr"/>
     </row>
@@ -4667,13 +4667,13 @@
         <v>234.717</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>274.968</v>
+        <v>328.471</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>1417.871</v>
+        <v>1254.701</v>
       </c>
       <c r="L55" t="inlineStr"/>
     </row>
@@ -4707,13 +4707,13 @@
         <v>234.717</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>274.968</v>
+        <v>328.471</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>1417.871</v>
+        <v>1254.701</v>
       </c>
       <c r="L56" t="inlineStr"/>
     </row>
@@ -4747,13 +4747,13 @@
         <v>234.717</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>274.968</v>
+        <v>328.471</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>1417.871</v>
+        <v>1254.701</v>
       </c>
       <c r="L57" t="inlineStr"/>
     </row>
@@ -4787,13 +4787,13 @@
         <v>234.717</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>274.967</v>
+        <v>328.47</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>1417.872</v>
+        <v>1254.702</v>
       </c>
       <c r="L58" t="inlineStr"/>
     </row>
@@ -4827,13 +4827,13 @@
         <v>234.717</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>274.968</v>
+        <v>328.471</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>1417.871</v>
+        <v>1254.701</v>
       </c>
       <c r="L59" t="inlineStr"/>
     </row>
@@ -4867,13 +4867,13 @@
         <v>234.717</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>274.968</v>
+        <v>328.471</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>1417.871</v>
+        <v>1254.701</v>
       </c>
       <c r="L60" t="inlineStr"/>
     </row>
@@ -4907,13 +4907,13 @@
         <v>234.717</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>274.967</v>
+        <v>328.47</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>1417.872</v>
+        <v>1254.702</v>
       </c>
       <c r="L61" t="inlineStr"/>
     </row>
@@ -4947,13 +4947,13 @@
         <v>234.717</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>274.967</v>
+        <v>328.47</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>1417.872</v>
+        <v>1254.702</v>
       </c>
       <c r="L62" t="inlineStr"/>
     </row>
@@ -4987,13 +4987,13 @@
         <v>234.717</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>274.968</v>
+        <v>328.471</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>1417.871</v>
+        <v>1254.701</v>
       </c>
       <c r="L63" t="inlineStr"/>
     </row>
@@ -5027,13 +5027,13 @@
         <v>234.717</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>274.968</v>
+        <v>328.471</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>1417.871</v>
+        <v>1254.701</v>
       </c>
       <c r="L64" t="inlineStr"/>
     </row>
@@ -5067,13 +5067,13 @@
         <v>234.717</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>274.968</v>
+        <v>328.471</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>1417.871</v>
+        <v>1254.701</v>
       </c>
       <c r="L65" t="inlineStr"/>
     </row>
@@ -5107,13 +5107,13 @@
         <v>234.717</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>274.967</v>
+        <v>328.47</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>1417.872</v>
+        <v>1254.702</v>
       </c>
       <c r="L66" t="inlineStr"/>
     </row>
@@ -5147,13 +5147,13 @@
         <v>234.717</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>274.968</v>
+        <v>328.471</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>1417.871</v>
+        <v>1254.701</v>
       </c>
       <c r="L67" t="inlineStr"/>
     </row>
@@ -5187,13 +5187,13 @@
         <v>234.717</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>274.967</v>
+        <v>328.47</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>1417.872</v>
+        <v>1254.702</v>
       </c>
       <c r="L68" t="inlineStr"/>
     </row>
@@ -5227,13 +5227,13 @@
         <v>234.717</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>274.967</v>
+        <v>328.47</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>1417.872</v>
+        <v>1254.702</v>
       </c>
       <c r="L69" t="inlineStr"/>
     </row>
@@ -5267,13 +5267,13 @@
         <v>234.717</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>274.968</v>
+        <v>328.471</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>1417.871</v>
+        <v>1254.701</v>
       </c>
       <c r="L70" t="inlineStr"/>
     </row>
@@ -5307,13 +5307,13 @@
         <v>234.717</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>274.968</v>
+        <v>328.471</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>1417.871</v>
+        <v>1254.701</v>
       </c>
       <c r="L71" t="inlineStr"/>
     </row>
@@ -5347,13 +5347,13 @@
         <v>234.717</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>274.968</v>
+        <v>328.471</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>1417.871</v>
+        <v>1254.701</v>
       </c>
       <c r="L72" t="inlineStr"/>
     </row>
@@ -5387,13 +5387,13 @@
         <v>234.717</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>274.968</v>
+        <v>328.471</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K73" s="2" t="n">
-        <v>1417.871</v>
+        <v>1254.701</v>
       </c>
       <c r="L73" t="inlineStr"/>
     </row>
@@ -5427,13 +5427,13 @@
         <v>234.717</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>274.968</v>
+        <v>328.471</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>1417.871</v>
+        <v>1254.701</v>
       </c>
       <c r="L74" t="inlineStr"/>
     </row>
@@ -5467,13 +5467,13 @@
         <v>234.717</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>274.968</v>
+        <v>328.471</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>1417.871</v>
+        <v>1254.701</v>
       </c>
       <c r="L75" t="inlineStr"/>
     </row>
@@ -5507,13 +5507,13 @@
         <v>234.717</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>274.968</v>
+        <v>328.471</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>1165.69</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>1417.871</v>
+        <v>1254.701</v>
       </c>
       <c r="L76" t="inlineStr"/>
     </row>
@@ -5547,13 +5547,13 @@
         <v>230.37</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>268.925</v>
+        <v>300.209</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>937.135</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>1091.987</v>
+        <v>971.308</v>
       </c>
       <c r="L77" t="inlineStr"/>
     </row>
@@ -5587,13 +5587,13 @@
         <v>230.37</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>268.924</v>
+        <v>300.209</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>937.135</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>1091.988</v>
+        <v>971.308</v>
       </c>
       <c r="L78" t="inlineStr"/>
     </row>
@@ -5627,13 +5627,13 @@
         <v>230.37</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>268.924</v>
+        <v>300.209</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>937.135</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>1091.988</v>
+        <v>971.308</v>
       </c>
       <c r="L79" t="inlineStr"/>
     </row>
@@ -5667,13 +5667,13 @@
         <v>230.37</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>268.924</v>
+        <v>300.209</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>937.135</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>1091.988</v>
+        <v>971.308</v>
       </c>
       <c r="L80" t="inlineStr"/>
     </row>
@@ -5707,13 +5707,13 @@
         <v>230.37</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>268.925</v>
+        <v>300.209</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>937.135</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>1091.987</v>
+        <v>971.308</v>
       </c>
       <c r="L81" t="inlineStr"/>
     </row>
@@ -5747,13 +5747,13 @@
         <v>230.37</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>268.925</v>
+        <v>300.209</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>937.135</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>1091.987</v>
+        <v>971.308</v>
       </c>
       <c r="L82" t="inlineStr"/>
     </row>
@@ -5787,13 +5787,13 @@
         <v>230.37</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>268.925</v>
+        <v>300.209</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>937.135</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>1091.987</v>
+        <v>971.308</v>
       </c>
       <c r="L83" t="inlineStr"/>
     </row>
@@ -5827,13 +5827,13 @@
         <v>230.37</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>268.925</v>
+        <v>300.209</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>937.135</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>1091.987</v>
+        <v>971.308</v>
       </c>
       <c r="L84" t="inlineStr"/>
     </row>
@@ -5867,13 +5867,13 @@
         <v>230.37</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>268.925</v>
+        <v>300.209</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>937.135</v>
       </c>
       <c r="K85" s="2" t="n">
-        <v>1091.987</v>
+        <v>971.308</v>
       </c>
       <c r="L85" t="inlineStr"/>
     </row>
@@ -5907,13 +5907,13 @@
         <v>227.762</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>265.3</v>
+        <v>298.313</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>822.8579999999999</v>
       </c>
       <c r="K86" s="2" t="n">
-        <v>890.429</v>
+        <v>778.312</v>
       </c>
       <c r="L86" t="inlineStr"/>
     </row>
@@ -5947,13 +5947,13 @@
         <v>227.762</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>265.3</v>
+        <v>298.313</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>822.8579999999999</v>
       </c>
       <c r="K87" s="2" t="n">
-        <v>890.429</v>
+        <v>778.312</v>
       </c>
       <c r="L87" t="inlineStr"/>
     </row>
@@ -5987,13 +5987,13 @@
         <v>227.762</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>265.299</v>
+        <v>298.312</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>822.8579999999999</v>
       </c>
       <c r="K88" s="2" t="n">
-        <v>890.4299999999999</v>
+        <v>778.313</v>
       </c>
       <c r="L88" t="inlineStr"/>
     </row>
@@ -6027,13 +6027,13 @@
         <v>227.762</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>265.299</v>
+        <v>298.312</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>822.8579999999999</v>
       </c>
       <c r="K89" s="2" t="n">
-        <v>890.4299999999999</v>
+        <v>778.313</v>
       </c>
       <c r="L89" t="inlineStr"/>
     </row>
@@ -6067,13 +6067,13 @@
         <v>227.762</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>265.3</v>
+        <v>298.313</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>822.8579999999999</v>
       </c>
       <c r="K90" s="2" t="n">
-        <v>890.429</v>
+        <v>778.312</v>
       </c>
       <c r="L90" t="inlineStr"/>
     </row>
@@ -6107,13 +6107,13 @@
         <v>227.762</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>265.3</v>
+        <v>298.313</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>822.8579999999999</v>
       </c>
       <c r="K91" s="2" t="n">
-        <v>890.429</v>
+        <v>778.312</v>
       </c>
       <c r="L91" t="inlineStr"/>
     </row>
@@ -6147,13 +6147,13 @@
         <v>227.762</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>265.3</v>
+        <v>298.313</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>822.8579999999999</v>
       </c>
       <c r="K92" s="2" t="n">
-        <v>890.429</v>
+        <v>778.312</v>
       </c>
       <c r="L92" t="inlineStr"/>
     </row>
@@ -6187,13 +6187,13 @@
         <v>227.762</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>265.3</v>
+        <v>298.313</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>822.8579999999999</v>
       </c>
       <c r="K93" s="2" t="n">
-        <v>890.429</v>
+        <v>778.312</v>
       </c>
       <c r="L93" t="inlineStr"/>
     </row>
@@ -6227,13 +6227,13 @@
         <v>227.762</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>265.3</v>
+        <v>298.313</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>822.8579999999999</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>890.429</v>
+        <v>778.312</v>
       </c>
       <c r="L94" t="inlineStr"/>
     </row>
@@ -6267,13 +6267,13 @@
         <v>226.024</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>262.884</v>
+        <v>284.768</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>728.747</v>
       </c>
       <c r="K95" s="2" t="n">
-        <v>760.974</v>
+        <v>668.369</v>
       </c>
       <c r="L95" t="inlineStr"/>
     </row>
@@ -6307,13 +6307,13 @@
         <v>226.024</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>262.884</v>
+        <v>284.768</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>728.747</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>760.974</v>
+        <v>668.369</v>
       </c>
       <c r="L96" t="inlineStr"/>
     </row>
@@ -6347,13 +6347,13 @@
         <v>226.024</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>262.884</v>
+        <v>284.768</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>728.747</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>760.974</v>
+        <v>668.369</v>
       </c>
       <c r="L97" t="inlineStr"/>
     </row>
@@ -6387,13 +6387,13 @@
         <v>223.02</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>258.709</v>
+        <v>251.783</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>564.665</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>541.62</v>
+        <v>493.502</v>
       </c>
       <c r="L98" t="inlineStr"/>
     </row>
@@ -6427,13 +6427,13 @@
         <v>222.716</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>258.285</v>
+        <v>249.828</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>548.165</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>518.739</v>
+        <v>473.566</v>
       </c>
       <c r="L99" t="inlineStr"/>
     </row>
@@ -6467,13 +6467,13 @@
         <v>221.282</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>256.292</v>
+        <v>240.636</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>470.554</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>411.12</v>
+        <v>379.794</v>
       </c>
       <c r="L100" t="inlineStr"/>
     </row>
@@ -6507,13 +6507,13 @@
         <v>221.282</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>256.292</v>
+        <v>240.636</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>470.554</v>
       </c>
       <c r="K101" s="2" t="n">
-        <v>411.12</v>
+        <v>379.794</v>
       </c>
       <c r="L101" t="inlineStr"/>
     </row>
@@ -6547,13 +6547,13 @@
         <v>220.593</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>255.335</v>
+        <v>236.22</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>433.276</v>
       </c>
       <c r="K102" s="2" t="n">
-        <v>359.426</v>
+        <v>334.754</v>
       </c>
       <c r="L102" t="inlineStr"/>
     </row>
@@ -6587,13 +6587,13 @@
         <v>219.423</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>253.709</v>
+        <v>233.27</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>432.072</v>
       </c>
       <c r="K103" s="2" t="n">
-        <v>269.781</v>
+        <v>250.914</v>
       </c>
       <c r="L103" t="inlineStr"/>
     </row>
@@ -6627,13 +6627,13 @@
         <v>218.239</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>252.063</v>
+        <v>224.346</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>357.285</v>
       </c>
       <c r="K104" s="2" t="n">
-        <v>181.548</v>
+        <v>175.653</v>
       </c>
       <c r="L104" t="inlineStr"/>
     </row>
@@ -6667,13 +6667,13 @@
         <v>217.25</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>250.688</v>
+        <v>215.922</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>289.225</v>
       </c>
       <c r="K105" s="2" t="n">
-        <v>107.966</v>
+        <v>114.198</v>
       </c>
       <c r="L105" t="inlineStr"/>
     </row>
@@ -6707,13 +6707,13 @@
         <v>217.25</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>250.687</v>
+        <v>215.921</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>289.225</v>
       </c>
       <c r="K106" s="2" t="n">
-        <v>107.967</v>
+        <v>114.199</v>
       </c>
       <c r="L106" t="inlineStr"/>
     </row>
@@ -6747,13 +6747,13 @@
         <v>216.895</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>250.194</v>
+        <v>213.264</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>265.924</v>
       </c>
       <c r="K107" s="2" t="n">
-        <v>81.53400000000001</v>
+        <v>91.652</v>
       </c>
       <c r="L107" t="inlineStr"/>
     </row>
@@ -6787,13 +6787,13 @@
         <v>216.5</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>249.646</v>
+        <v>210.381</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>237.966</v>
       </c>
       <c r="K108" s="2" t="n">
-        <v>52.014</v>
+        <v>66.337</v>
       </c>
       <c r="L108" t="inlineStr"/>
     </row>
@@ -6827,13 +6827,13 @@
         <v>201.666</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>201.666</v>
+        <v>161.333</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>157.299</v>
       </c>
       <c r="K109" s="2" t="n">
-        <v>0</v>
+        <v>20.167</v>
       </c>
       <c r="L109" t="inlineStr">
         <is>
@@ -6871,13 +6871,13 @@
         <v>201.666</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>201.666</v>
+        <v>161.333</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>157.299</v>
       </c>
       <c r="K110" s="2" t="n">
-        <v>0</v>
+        <v>20.167</v>
       </c>
       <c r="L110" t="inlineStr">
         <is>
@@ -6915,13 +6915,13 @@
         <v>201.666</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>201.666</v>
+        <v>161.333</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>157.299</v>
       </c>
       <c r="K111" s="2" t="n">
-        <v>0</v>
+        <v>20.167</v>
       </c>
       <c r="L111" t="inlineStr">
         <is>
@@ -6959,13 +6959,13 @@
         <v>201.666</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>201.666</v>
+        <v>161.333</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>157.299</v>
       </c>
       <c r="K112" s="2" t="n">
-        <v>0</v>
+        <v>20.167</v>
       </c>
       <c r="L112" t="inlineStr">
         <is>
@@ -7003,13 +7003,13 @@
         <v>201.666</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>201.666</v>
+        <v>161.333</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>157.299</v>
       </c>
       <c r="K113" s="2" t="n">
-        <v>0</v>
+        <v>20.167</v>
       </c>
       <c r="L113" t="inlineStr">
         <is>
@@ -7047,13 +7047,13 @@
         <v>201.666</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>201.666</v>
+        <v>161.333</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>157.299</v>
       </c>
       <c r="K114" s="2" t="n">
-        <v>0</v>
+        <v>20.167</v>
       </c>
       <c r="L114" t="inlineStr">
         <is>
@@ -7091,13 +7091,13 @@
         <v>201.666</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>201.666</v>
+        <v>161.333</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>157.299</v>
       </c>
       <c r="K115" s="2" t="n">
-        <v>0</v>
+        <v>20.167</v>
       </c>
       <c r="L115" t="inlineStr">
         <is>
@@ -7135,13 +7135,13 @@
         <v>201.666</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>201.666</v>
+        <v>161.333</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>157.299</v>
       </c>
       <c r="K116" s="2" t="n">
-        <v>0</v>
+        <v>20.167</v>
       </c>
       <c r="L116" t="inlineStr">
         <is>
@@ -7179,13 +7179,13 @@
         <v>164.999</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>164.999</v>
+        <v>131.999</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>137.193</v>
       </c>
       <c r="K117" s="2" t="n">
-        <v>0</v>
+        <v>16.5</v>
       </c>
       <c r="L117" t="inlineStr">
         <is>
@@ -7223,13 +7223,13 @@
         <v>0</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>0</v>
+        <v>77.008</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>725.997</v>
       </c>
       <c r="K118" s="2" t="n">
-        <v>791.202</v>
+        <v>661.596</v>
       </c>
       <c r="L118" t="inlineStr"/>
     </row>
@@ -7263,13 +7263,13 @@
         <v>0</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>0</v>
+        <v>94.809</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>922.533</v>
       </c>
       <c r="K119" s="2" t="n">
-        <v>1027.395</v>
+        <v>866.23</v>
       </c>
       <c r="L119" t="inlineStr"/>
     </row>
@@ -7303,13 +7303,13 @@
         <v>0</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>0</v>
+        <v>133.154</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>1245.287</v>
       </c>
       <c r="K120" s="2" t="n">
-        <v>1386.42</v>
+        <v>1162.066</v>
       </c>
       <c r="L120" t="inlineStr"/>
     </row>
@@ -7343,13 +7343,13 @@
         <v>0</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>0</v>
+        <v>39.316</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>396.671</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>426.361</v>
+        <v>359.266</v>
       </c>
       <c r="L121" t="inlineStr"/>
     </row>
@@ -7364,7 +7364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -7416,7 +7416,7 @@
         <v>890.355</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>169.761</v>
+        <v>696.605</v>
       </c>
     </row>
     <row r="4">
@@ -7429,7 +7429,7 @@
         <v>2834.781</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>8258.596</v>
+        <v>6982.731</v>
       </c>
     </row>
     <row r="5">
@@ -7442,7 +7442,7 @@
         <v>417.265</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>42.125</v>
+        <v>684.774</v>
       </c>
     </row>
     <row r="6">
@@ -7481,7 +7481,7 @@
         <v>0</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>5339.947</v>
+        <v>5446.319</v>
       </c>
     </row>
     <row r="9">
@@ -7507,175 +7507,188 @@
         <v>0</v>
       </c>
       <c r="C10" s="2" t="n">
+        <v>3504.669</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CostBucketOverheadsImaging</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>122.89</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>CostBucketOverheads TOTAL</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="2" t="n">
         <v>3627.559</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>CostBucketOverheads TOTAL</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="2" t="n">
-        <v>3627.559</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>CostTypeDetailsDepreciation</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>348.76</v>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>221.721</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CostTypeDetailsMS</t>
+          <t>CostTypeDetailsDepreciation</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>1111.882</v>
+        <v>348.76</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>602.0410000000001</v>
+        <v>221.721</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CostTypeDetailsOHC</t>
+          <t>CostTypeDetailsMS</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>175.999</v>
+        <v>1111.882</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>1117.688</v>
+        <v>602.0410000000001</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CostTypeDetailsOHDepreciation</t>
+          <t>CostTypeDetailsOHC</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0</v>
+        <v>175.999</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>52.068</v>
+        <v>1117.688</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CostTypeDetailsOHF</t>
+          <t>CostTypeDetailsOHDepreciation</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>524.759</v>
+        <v>0</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>2457.803</v>
+        <v>52.068</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CostTypeDetailsPharmacy</t>
+          <t>CostTypeDetailsOHF</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>0</v>
+        <v>524.759</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>29.198</v>
+        <v>2457.803</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CostTypeDetailsProstheses</t>
+          <t>CostTypeDetailsPharmacy</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>5080.522</v>
+        <v>29.198</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CostTypeDetailsSWAllied</t>
+          <t>CostTypeDetailsProstheses</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>695.472</v>
+        <v>0</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>433.091</v>
+        <v>5080.522</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CostTypeDetailsSWDoc</t>
+          <t>CostTypeDetailsSWAllied</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>7066.556</v>
+        <v>695.472</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>6612.445</v>
+        <v>433.091</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CostTypeDetailsSWNonClin</t>
+          <t>CostTypeDetailsSWDoc</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>871.899</v>
+        <v>7066.556</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>0</v>
+        <v>6612.445</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>CostTypeDetailsSWNonClin</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>871.899</v>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>CostTypeDetailsSWNurs</t>
         </is>
       </c>
-      <c r="B22" s="2" t="n">
+      <c r="B23" s="2" t="n">
         <v>2396.066</v>
       </c>
-      <c r="C22" s="2" t="n">
+      <c r="C23" s="2" t="n">
         <v>831.4109999999999</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
         <is>
           <t>CostTypeDetails TOTAL</t>
         </is>
       </c>
-      <c r="B23" s="2" t="n">
+      <c r="B24" s="2" t="n">
         <v>13191.393</v>
       </c>
-      <c r="C23" s="2" t="n">
+      <c r="C24" s="2" t="n">
         <v>17437.988</v>
       </c>
     </row>
@@ -7690,7 +7703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A262"/>
+  <dimension ref="A1:A250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -7902,1631 +7915,1547 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Prosthesis profile SWAllied 13.0%, Prostheses 87.0%</t>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Prosthesis profile SWNurs 3.6%, SWDoc 29.5%, SWAllied 11.1%, Prostheses 54.3%, MS 1.5%</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Dental profile SWNurs 8.2%, SWDoc 47.0%, SWAllied 2.4%, MS 7.5%, GS 0.2%, Depreciation 2.4%, OHF 29.7%, OHDepreciation 0.6%, OHC 2.0%</t>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Dental profile SWNurs 8.1%, SWDoc 41.8%, SWAllied 2.2%, Prostheses 1.9%, MS 7.4%, GS 0.3%, Depreciation 2.6%, OHF 32.7%, OHDepreciation 0.7%, OHC 2.3%</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Anaesthesia profile SWNurs 6.5%, SWDoc 71.5%, Pharmacy 22.1%</t>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Imaging profile SWNurs 7.4%, SWDoc 40.7%, SWAllied 4.1%, Prostheses 14.1%, MS 6.4%, Depreciation 2.1%, OHF 25.2%</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Imaging profile SWNurs 77.7%, Depreciation 22.3%</t>
+          <t>CostSubmission_MF4159_2025_M01_PROD.xml: bucket Anaesthesia profile SWNurs 9.7%, SWDoc 53.8%, Pharmacy 6.6%, Prostheses 18.6%, MS 8.4%, Depreciation 2.8%</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">CostSubmission_MF4159_2025_M01_PROD.xml: bucket Laboratory profile </t>
+          <t>CostSubmission_MF4159_2025_M02_PROD.xml: claim totals -0.015 AED vs ledger absorbed by claim 760MF4159-03a04e</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M02_PROD.xml: claim totals -0.015 AED vs ledger absorbed by claim 760MF4159-03a04e</t>
+          <t>CostSubmission_MF4159_2025_M02_PROD.xml: Prostheses pools abutments 4,275.00, bone_graft 9,150.00, fixtures 29,846.00, lab 15,958.44; coded claims in activity: 127</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M02_PROD.xml: Prostheses pools abutments 4,275.00, bone_graft 9,150.00, fixtures 29,846.00, lab 15,958.44; coded claims in activity: 127</t>
+          <t>CostSubmission_MF4159_2025_M02_PROD.xml: abutments pool 4,275.000 AED placed on 15 claims by units (36 units; 118.750 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M02_PROD.xml: abutments pool 4,275.000 AED placed on 15 claims by units (36 units; 118.750 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M02_PROD.xml: bone_graft pool 9,150.000 AED placed on 20 claims by units (70 units; 130.714 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M02_PROD.xml: bone_graft pool 9,150.000 AED placed on 20 claims by units (70 units; 130.714 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M02_PROD.xml: fixtures pool 29,846.000 AED placed on 15 claims by units (32 units; 932.688 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M02_PROD.xml: fixtures pool 29,846.000 AED placed on 15 claims by units (32 units; 932.688 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M02_PROD.xml: lab pool 15,958.440 AED placed on 127 claims by units (330 units; 48.359 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M02_PROD.xml: lab pool 15,958.440 AED placed on 127 claims by units (330 units; 48.359 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M02_PROD.xml: dental technicians pool 6,666.308 AED placed on 127 claims by units (330 units; 20.201 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M02_PROD.xml: dental technicians pool 6,666.308 AED placed on 127 claims by units (330 units; 20.201 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M02_PROD.xml: fils residuals {SWNurs:-19, SWDoc:+4, SWAllied:+17, Pharmacy:+36, MS:-64, GS:-23, Depreciation:+46, OHF:+17, OHDepreciation:+32, OHC:-46} absorbed by claim index 815</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M02_PROD.xml: fils residuals {SWNurs:-19, SWDoc:+4, SWAllied:+17, Pharmacy:+36, MS:-64, GS:-23, Depreciation:+46, OHF:+17, OHDepreciation:+32, OHC:-46} absorbed by claim index 815</t>
+          <t>CostSubmission_MF4159_2025_M02_PROD.xml: bucket Prosthesis profile SWNurs 3.1%, SWDoc 37.9%, SWAllied 7.9%, Prostheses 49.6%, MS 1.5%</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M02_PROD.xml: bucket Prosthesis profile SWAllied 10.1%, Prostheses 89.9%</t>
+          <t>CostSubmission_MF4159_2025_M02_PROD.xml: bucket Dental profile SWNurs 6.1%, SWDoc 46.0%, SWAllied 1.7%, Prostheses 1.5%, MS 6.1%, GS 0.6%, Depreciation 2.4%, OHF 25.4%, OHDepreciation 0.6%, OHC 9.5%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M02_PROD.xml: bucket Dental profile SWNurs 6.2%, SWDoc 51.5%, SWAllied 1.8%, MS 6.2%, GS 0.5%, Depreciation 2.2%, OHF 22.9%, OHDepreciation 0.6%, OHC 8.1%</t>
+          <t>CostSubmission_MF4159_2025_M02_PROD.xml: bucket Imaging profile SWNurs 6.1%, SWDoc 49.1%, SWAllied 3.4%, Prostheses 12.1%, MS 5.8%, Depreciation 2.2%, OHF 21.4%</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M02_PROD.xml: bucket Anaesthesia profile SWNurs 4.8%, SWDoc 77.5%, Pharmacy 17.7%</t>
+          <t>CostSubmission_MF4159_2025_M02_PROD.xml: bucket Anaesthesia profile SWNurs 7.7%, SWDoc 61.6%, Pharmacy 5.6%, Prostheses 15.1%, MS 7.3%, Depreciation 2.7%</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M02_PROD.xml: bucket Imaging profile SWNurs 74.0%, Depreciation 26.0%</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: claim totals -0.047 AED vs ledger absorbed by claim 1776MF4159-ea919c</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">CostSubmission_MF4159_2025_M02_PROD.xml: bucket Laboratory profile </t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: Prostheses pools bone_graft 7,850.00, fixtures 22,483.00, abutments 9,790.00, lab 48,028.42; coded claims in activity: 116</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: claim totals -0.047 AED vs ledger absorbed by claim 1776MF4159-ea919c</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: bone_graft pool 7,850.000 AED placed on 11 claims by units (32 units; 245.312 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: Prostheses pools bone_graft 7,850.00, fixtures 22,483.00, abutments 9,790.00, lab 48,028.42; coded claims in activity: 116</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: fixtures pool 22,483.000 AED placed on 12 claims by units (17 units; 1,322.529 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: bone_graft pool 7,850.000 AED placed on 11 claims by units (32 units; 245.312 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: abutments: claim 781MF4159-26d379 share 391.600 capped at its Dental amount 302.499</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: fixtures pool 22,483.000 AED placed on 12 claims by units (17 units; 1,322.529 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: abutments: claim 2661MF4159-d5af2d share 391.600 capped at its Dental amount 302.499</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: abutments: claim 781MF4159-26d379 share 391.600 capped at its Dental amount 302.499</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: abutments: claim 1337MF4159-ecf85b share 391.600 capped at its Dental amount 302.499</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: abutments: claim 2661MF4159-d5af2d share 391.600 capped at its Dental amount 302.499</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: abutments: claim 2669MF4159-56bb2c share 391.600 capped at its Dental amount 302.499</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: abutments: claim 1337MF4159-ecf85b share 391.600 capped at its Dental amount 302.499</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: abutments: claim 2436MF4159-aa32a4 share 391.600 capped at its Dental amount 302.499</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: abutments: claim 2669MF4159-56bb2c share 391.600 capped at its Dental amount 302.499</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: abutments: claim 1792MF4159-adecc5 share 783.200 capped at its Dental amount 635.553</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: abutments: claim 2436MF4159-aa32a4 share 391.600 capped at its Dental amount 302.499</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: abutments: claim 1941MF4159-15afa4 share 391.600 capped at its Dental amount 164.999</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: abutments: claim 1792MF4159-adecc5 share 783.200 capped at its Dental amount 635.553</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: abutments: claim 2346MF4159-af3dfb share 1,566.400 capped at its Dental amount 1,209.995</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: abutments: claim 1941MF4159-15afa4 share 391.600 capped at its Dental amount 164.999</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: abutments: claim 1790MF4159-305d29 share 391.600 capped at its Dental amount 302.499</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: abutments: claim 2346MF4159-af3dfb share 1,566.400 capped at its Dental amount 1,209.995</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: abutments pool 9,790.000 AED placed on 18 claims by units (25 units; 391.600 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: abutments: claim 1790MF4159-305d29 share 391.600 capped at its Dental amount 302.499</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 697MF4159-2ac13e share 215.374 capped at its Dental amount 201.666</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: abutments pool 9,790.000 AED placed on 18 claims by units (25 units; 391.600 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 781MF4159-26d379 share 215.374 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 697MF4159-2ac13e share 215.374 capped at its Dental amount 201.666</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 2646MF4159-7976bf share 215.374 capped at its Dental amount 201.666</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 781MF4159-26d379 share 215.374 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 615MF4159-c15e63 share 215.374 capped at its Dental amount 201.666</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 2646MF4159-7976bf share 215.374 capped at its Dental amount 201.666</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 2661MF4159-d5af2d share 215.374 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 615MF4159-c15e63 share 215.374 capped at its Dental amount 201.666</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1337MF4159-ecf85b share 215.374 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 2661MF4159-d5af2d share 215.374 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 2669MF4159-56bb2c share 215.374 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1337MF4159-ecf85b share 215.374 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1900MF4159-6f3eb9 share 215.374 capped at its Dental amount 201.666</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 2669MF4159-56bb2c share 215.374 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 2436MF4159-aa32a4 share 215.374 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1900MF4159-6f3eb9 share 215.374 capped at its Dental amount 201.666</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1736MF4159-c8f10a share 1,292.245 capped at its Dental amount 1,209.995</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 2436MF4159-aa32a4 share 215.374 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1792MF4159-adecc5 share 430.748 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1736MF4159-c8f10a share 1,292.245 capped at its Dental amount 1,209.995</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1941MF4159-15afa4 share 215.374 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1792MF4159-adecc5 share 430.748 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 2346MF4159-af3dfb share 861.497 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1941MF4159-15afa4 share 215.374 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1635MF4159-e561c4 share 1,507.619 capped at its Dental amount 1,411.661</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 2346MF4159-af3dfb share 861.497 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1978MF4159-7c60ba share 215.374 capped at its Dental amount 201.666</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1635MF4159-e561c4 share 1,507.619 capped at its Dental amount 1,411.661</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1790MF4159-305d29 share 215.374 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1978MF4159-7c60ba share 215.374 capped at its Dental amount 201.666</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1886MF4159-cb3d3f share 215.374 capped at its Dental amount 201.666</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1790MF4159-305d29 share 215.374 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1981MF4159-97470b share 215.374 capped at its Dental amount 201.666</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1886MF4159-cb3d3f share 215.374 capped at its Dental amount 201.666</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1971MF4159-abc46a share 430.748 capped at its Dental amount 403.332</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1981MF4159-97470b share 215.374 capped at its Dental amount 201.666</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1992MF4159-7be120 share 215.374 capped at its Dental amount 201.666</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1971MF4159-abc46a share 430.748 capped at its Dental amount 403.332</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab pool 48,028.420 AED placed on 107 claims by units (223 units; 215.374 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab: claim 1992MF4159-7be120 share 215.374 capped at its Dental amount 201.666</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 697MF4159-2ac13e share 32.875 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: lab pool 48,028.420 AED placed on 107 claims by units (223 units; 215.374 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 781MF4159-26d379 share 32.875 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 697MF4159-2ac13e share 32.875 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 2646MF4159-7976bf share 32.875 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 781MF4159-26d379 share 32.875 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 615MF4159-c15e63 share 32.875 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 2646MF4159-7976bf share 32.875 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 2661MF4159-d5af2d share 32.875 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 615MF4159-c15e63 share 32.875 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1337MF4159-ecf85b share 32.875 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 2661MF4159-d5af2d share 32.875 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 2669MF4159-56bb2c share 32.875 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1337MF4159-ecf85b share 32.875 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1900MF4159-6f3eb9 share 32.875 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 2669MF4159-56bb2c share 32.875 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 2436MF4159-aa32a4 share 32.875 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1900MF4159-6f3eb9 share 32.875 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1736MF4159-c8f10a share 197.248 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 2436MF4159-aa32a4 share 32.875 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1792MF4159-adecc5 share 65.749 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1736MF4159-c8f10a share 197.248 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1941MF4159-15afa4 share 32.875 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1792MF4159-adecc5 share 65.749 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 2346MF4159-af3dfb share 131.498 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1941MF4159-15afa4 share 32.875 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1635MF4159-e561c4 share 230.122 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 2346MF4159-af3dfb share 131.498 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1978MF4159-7c60ba share 32.874 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1635MF4159-e561c4 share 230.122 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1790MF4159-305d29 share 32.874 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1978MF4159-7c60ba share 32.874 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1886MF4159-cb3d3f share 32.874 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1790MF4159-305d29 share 32.874 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1981MF4159-97470b share 32.874 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1886MF4159-cb3d3f share 32.874 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1971MF4159-abc46a share 65.749 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1981MF4159-97470b share 32.874 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1992MF4159-7be120 share 32.874 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1971MF4159-abc46a share 65.749 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians pool 7,331.045 AED placed on 96 claims by units (223 units; 32.875 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians: claim 1992MF4159-7be120 share 32.874 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: fils residuals {SWNurs:-67, SWDoc:+2, SWAllied:+57, Pharmacy:+34, MS:-31, Depreciation:-25, OHF:+47, OHDepreciation:+1, OHC:-18} absorbed by claim index 180</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: dental technicians pool 7,331.045 AED placed on 96 claims by units (223 units; 32.875 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: bucket Prosthesis profile SWNurs 2.7%, SWDoc 30.2%, SWAllied 6.9%, Prostheses 58.9%, MS 1.3%</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: fils residuals {SWNurs:-67, SWDoc:+2, SWAllied:+57, Pharmacy:+34, MS:-31, Depreciation:-25, OHF:+47, OHDepreciation:+1, OHC:-18} absorbed by claim index 180</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: bucket Dental profile SWNurs 5.9%, SWDoc 41.3%, SWAllied 1.7%, Prostheses 2.0%, MS 6.0%, Depreciation 2.2%, OHF 26.1%, OHDepreciation 0.6%, OHC 14.2%</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: bucket Prosthesis profile SWAllied 7.7%, Prostheses 92.3%</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: bucket Imaging profile SWNurs 6.0%, SWDoc 44.5%, SWAllied 3.4%, Prostheses 16.2%, MS 5.7%, Depreciation 1.9%, OHF 22.2%</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: bucket Dental profile SWNurs 6.2%, SWDoc 47.0%, SWAllied 1.8%, MS 6.2%, Depreciation 2.0%, OHF 24.0%, OHDepreciation 0.5%, OHC 12.4%</t>
+          <t>CostSubmission_MF4159_2025_M03_PROD.xml: bucket Anaesthesia profile SWNurs 7.7%, SWDoc 56.8%, Pharmacy 5.0%, Prostheses 20.7%, MS 7.3%, Depreciation 2.5%</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: bucket Anaesthesia profile SWNurs 5.2%, SWDoc 77.7%, Pharmacy 17.1%</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: claim totals -0.004 AED vs ledger absorbed by claim 1689MF4159-a7a492</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M03_PROD.xml: bucket Imaging profile SWNurs 75.5%, Depreciation 24.5%</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: Prostheses pools abutments 9,790.00, bone_graft 7,850.00, fixtures 22,483.00, lab 30,336.42; coded claims in activity: 138</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t xml:space="preserve">CostSubmission_MF4159_2025_M03_PROD.xml: bucket Laboratory profile </t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: abutments: claim 1474MF4159-6abc84 share 287.941 capped at its Dental amount 256.783</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: claim totals -0.004 AED vs ledger absorbed by claim 1689MF4159-a7a492</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: abutments: claim 1580MF4159-b18ada share 287.941 capped at its Dental amount 233.225</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: Prostheses pools abutments 9,790.00, bone_graft 7,850.00, fixtures 22,483.00, lab 30,336.42; coded claims in activity: 138</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: abutments: claim 2026MF4159-47d5d0 share 575.883 capped at its Dental amount 466.449</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: abutments: claim 1474MF4159-6abc84 share 287.941 capped at its Dental amount 256.783</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: abutments: claim 388MF4159-b700c3 share 287.941 capped at its Dental amount 233.225</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: abutments: claim 1580MF4159-b18ada share 287.941 capped at its Dental amount 233.225</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: abutments pool 9,790.000 AED placed on 17 claims by units (34 units; 287.941 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: abutments: claim 2026MF4159-47d5d0 share 575.883 capped at its Dental amount 466.449</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: bone_graft pool 7,850.000 AED placed on 10 claims by units (66 units; 118.939 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: abutments: claim 388MF4159-b700c3 share 287.941 capped at its Dental amount 233.225</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: fixtures pool 22,483.000 AED placed on 10 claims by units (33 units; 681.303 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: abutments pool 9,790.000 AED placed on 17 claims by units (34 units; 287.941 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: lab: claim 1474MF4159-6abc84 share 86.183 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: bone_graft pool 7,850.000 AED placed on 10 claims by units (66 units; 118.939 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: lab: claim 1580MF4159-b18ada share 86.183 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: fixtures pool 22,483.000 AED placed on 10 claims by units (33 units; 681.303 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: lab: claim 2026MF4159-47d5d0 share 172.366 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: lab: claim 1474MF4159-6abc84 share 86.183 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: lab: claim 388MF4159-b700c3 share 86.183 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: lab: claim 1580MF4159-b18ada share 86.183 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: lab pool 30,336.420 AED placed on 134 claims by units (352 units; 86.183 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: lab: claim 2026MF4159-47d5d0 share 172.366 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: dental technicians: claim 1474MF4159-6abc84 share 11.957 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: lab: claim 388MF4159-b700c3 share 86.183 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: dental technicians: claim 1580MF4159-b18ada share 11.957 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: lab pool 30,336.420 AED placed on 134 claims by units (352 units; 86.183 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: dental technicians: claim 2026MF4159-47d5d0 share 23.914 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: dental technicians: claim 1474MF4159-6abc84 share 11.957 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: dental technicians: claim 388MF4159-b700c3 share 11.957 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: dental technicians: claim 1580MF4159-b18ada share 11.957 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: dental technicians pool 4,208.914 AED placed on 134 claims by units (352 units; 11.957 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: dental technicians: claim 2026MF4159-47d5d0 share 23.914 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: fils residuals {SWNurs:-32, SWDoc:-50, SWAllied:-21, Pharmacy:+2, MS:+32, GS:+27, Depreciation:-1, OHF:+47, OHDepreciation:+30, OHC:-34} absorbed by claim index 243</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: dental technicians: claim 388MF4159-b700c3 share 11.957 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: bucket Prosthesis profile SWNurs 3.7%, SWDoc 27.0%, SWAllied 5.6%, Prostheses 62.0%, MS 1.7%</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: dental technicians pool 4,208.914 AED placed on 134 claims by units (352 units; 11.957 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: bucket Dental profile SWNurs 7.0%, SWDoc 31.7%, SWAllied 1.9%, Prostheses 1.8%, MS 6.8%, GS 0.2%, Depreciation 2.4%, OHF 30.4%, OHDepreciation 0.7%, OHC 17.1%</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: fils residuals {SWNurs:-32, SWDoc:-50, SWAllied:-21, Pharmacy:+2, MS:+32, GS:+27, Depreciation:-1, OHF:+47, OHDepreciation:+30, OHC:-34} absorbed by claim index 243</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: bucket Imaging profile SWNurs 7.5%, SWDoc 36.2%, SWAllied 4.0%, Prostheses 15.6%, MS 6.9%, Depreciation 2.3%, OHF 27.5%</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: bucket Prosthesis profile SWAllied 5.6%, Prostheses 94.4%</t>
+          <t>CostSubmission_MF4159_2025_M04_PROD.xml: bucket Anaesthesia profile SWNurs 10.3%, SWDoc 49.5%, Pharmacy 6.4%, Prostheses 21.3%, MS 9.4%, Depreciation 3.2%</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: bucket Dental profile SWNurs 7.4%, SWDoc 36.7%, SWAllied 2.1%, MS 7.1%, GS 0.2%, Depreciation 2.3%, OHF 28.5%, OHDepreciation 0.6%, OHC 15.2%</t>
+          <t>CostSubmission_MF4159_2025_M05_PROD.xml: claim totals -0.037 AED vs ledger absorbed by claim 1351MF4159-60207a</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: bucket Anaesthesia profile SWNurs 7.3%, SWDoc 70.0%, Pharmacy 22.7%</t>
+          <t>CostSubmission_MF4159_2025_M05_PROD.xml: Prostheses pools bone_graft 8,935.00, fixtures 32,196.97, abutments 1,340.00, lab 21,167.08; coded claims in activity: 140</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M04_PROD.xml: bucket Imaging profile SWNurs 76.3%, Depreciation 23.7%</t>
+          <t>CostSubmission_MF4159_2025_M05_PROD.xml: bone_graft pool 8,935.000 AED placed on 20 claims by units (72 units; 124.097 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t xml:space="preserve">CostSubmission_MF4159_2025_M04_PROD.xml: bucket Laboratory profile </t>
+          <t>CostSubmission_MF4159_2025_M05_PROD.xml: fixtures pool 32,196.970 AED placed on 19 claims by units (38 units; 847.289 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M05_PROD.xml: claim totals -0.037 AED vs ledger absorbed by claim 1351MF4159-60207a</t>
+          <t>CostSubmission_MF4159_2025_M05_PROD.xml: abutments pool 1,340.000 AED placed on 21 claims by units (35 units; 38.286 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M05_PROD.xml: Prostheses pools bone_graft 8,935.00, fixtures 32,196.97, abutments 1,340.00, lab 21,167.08; coded claims in activity: 140</t>
+          <t>CostSubmission_MF4159_2025_M05_PROD.xml: lab pool 21,167.080 AED placed on 140 claims by units (319 units; 66.354 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M05_PROD.xml: bone_graft pool 8,935.000 AED placed on 20 claims by units (72 units; 124.097 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M05_PROD.xml: dental technicians pool 7,160.511 AED placed on 140 claims by units (319 units; 22.447 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M05_PROD.xml: fixtures pool 32,196.970 AED placed on 19 claims by units (38 units; 847.289 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M05_PROD.xml: fils residuals {SWNurs:-42, SWDoc:+8, SWAllied:-65, Pharmacy:-67, MS:+29, Depreciation:-20, OHF:+137, OHDepreciation:+65, OHC:-45} absorbed by claim index 54</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M05_PROD.xml: abutments pool 1,340.000 AED placed on 21 claims by units (35 units; 38.286 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M05_PROD.xml: bucket Prosthesis profile SWNurs 4.4%, SWDoc 30.8%, SWAllied 8.8%, Prostheses 54.7%, MS 1.3%</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M05_PROD.xml: lab pool 21,167.080 AED placed on 140 claims by units (319 units; 66.354 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M05_PROD.xml: bucket Dental profile SWNurs 9.2%, SWDoc 40.6%, SWAllied 2.3%, Prostheses 1.8%, MS 5.8%, Depreciation 2.7%, OHF 36.3%, OHDepreciation 0.7%, OHC 0.7%</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M05_PROD.xml: dental technicians pool 7,160.511 AED placed on 140 claims by units (319 units; 22.447 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M05_PROD.xml: bucket Imaging profile SWNurs 8.3%, SWDoc 39.4%, SWAllied 4.1%, Prostheses 13.1%, MS 5.0%, Depreciation 2.2%, OHF 27.8%</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M05_PROD.xml: fils residuals {SWNurs:-42, SWDoc:+8, SWAllied:-65, Pharmacy:-67, MS:+29, Depreciation:-20, OHF:+137, OHDepreciation:+65, OHC:-45} absorbed by claim index 54</t>
+          <t>CostSubmission_MF4159_2025_M05_PROD.xml: bucket Anaesthesia profile SWNurs 11.5%, SWDoc 54.2%, Pharmacy 6.5%, Prostheses 18.0%, MS 6.8%, Depreciation 3.0%</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M05_PROD.xml: bucket Prosthesis profile SWAllied 10.1%, Prostheses 89.9%</t>
+          <t>CostSubmission_MF4159_2025_M06_PROD.xml: claim totals +0.022 AED vs ledger absorbed by claim 165MF4159-98360e</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M05_PROD.xml: bucket Dental profile SWNurs 9.4%, SWDoc 45.7%, SWAllied 2.4%, MS 5.9%, Depreciation 2.5%, OHF 32.9%, OHDepreciation 0.6%, OHC 0.6%</t>
+          <t>CostSubmission_MF4159_2025_M06_PROD.xml: Prostheses pools fixtures 30,303.03, bone_graft 8,512.50, abutments 1,750.00, lab 12,441.50; coded claims in activity: 120</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M05_PROD.xml: bucket Anaesthesia profile SWNurs 7.5%, SWDoc 71.1%, Pharmacy 21.4%</t>
+          <t>CostSubmission_MF4159_2025_M06_PROD.xml: fixtures pool 30,303.030 AED placed on 15 claims by units (34 units; 891.266 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M05_PROD.xml: bucket Imaging profile SWNurs 79.3%, Depreciation 20.7%</t>
+          <t>CostSubmission_MF4159_2025_M06_PROD.xml: bone_graft pool 8,512.500 AED placed on 15 claims by units (66 units; 128.977 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t xml:space="preserve">CostSubmission_MF4159_2025_M05_PROD.xml: bucket Laboratory profile </t>
+          <t>CostSubmission_MF4159_2025_M06_PROD.xml: abutments pool 1,750.000 AED placed on 23 claims by units (33 units; 53.030 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M06_PROD.xml: claim totals +0.022 AED vs ledger absorbed by claim 165MF4159-98360e</t>
+          <t>CostSubmission_MF4159_2025_M06_PROD.xml: lab pool 12,441.500 AED placed on 120 claims by units (280 units; 44.434 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M06_PROD.xml: Prostheses pools fixtures 30,303.03, bone_graft 8,512.50, abutments 1,750.00, lab 12,441.50; coded claims in activity: 120</t>
+          <t>CostSubmission_MF4159_2025_M06_PROD.xml: fils residuals {SWNurs:+67, SWDoc:-59, SWAllied:+15, Pharmacy:-48, MS:+17, Depreciation:+41, OHF:+16, OHDepreciation:-64, OHC:+15} absorbed by claim index 419</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M06_PROD.xml: fixtures pool 30,303.030 AED placed on 15 claims by units (34 units; 891.266 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M06_PROD.xml: bucket Prosthesis profile SWNurs 6.9%, SWDoc 40.6%, SWAllied 1.7%, Prostheses 49.4%, MS 1.3%</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M06_PROD.xml: bone_graft pool 8,512.500 AED placed on 15 claims by units (66 units; 128.977 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M06_PROD.xml: bucket Dental profile SWNurs 9.8%, SWDoc 36.2%, SWAllied 2.5%, Prostheses 1.1%, MS 4.1%, Depreciation 2.0%, OHF 36.0%, OHDepreciation 0.5%, OHC 7.8%</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M06_PROD.xml: abutments pool 1,750.000 AED placed on 23 claims by units (33 units; 53.030 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M06_PROD.xml: bucket Imaging profile SWNurs 10.0%, SWDoc 39.4%, SWAllied 5.0%, Prostheses 9.0%, MS 3.9%, Depreciation 1.8%, OHF 30.9%</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M06_PROD.xml: lab pool 12,441.500 AED placed on 120 claims by units (280 units; 44.434 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M06_PROD.xml: bucket Anaesthesia profile SWNurs 14.9%, SWDoc 58.3%, Pharmacy 5.1%, Prostheses 13.3%, MS 5.8%, Depreciation 2.6%</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M06_PROD.xml: fils residuals {SWNurs:+67, SWDoc:-59, SWAllied:+15, Pharmacy:-48, MS:+17, Depreciation:+41, OHF:+16, OHDepreciation:-64, OHC:+15} absorbed by claim index 419</t>
+          <t>CostSubmission_MF4159_2025_M07_PROD.xml: claim totals -0.020 AED vs ledger absorbed by claim 2066MF4159-ff09af</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M06_PROD.xml: bucket Prosthesis profile Prostheses 100.0%</t>
+          <t>CostSubmission_MF4159_2025_M07_PROD.xml: Prostheses pools fixtures 14,810.61, abutments 6,350.00, bone_graft 5,800.00, lab 19,563.99; coded claims in activity: 122</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M06_PROD.xml: bucket Dental profile SWNurs 10.1%, SWDoc 41.1%, SWAllied 2.7%, MS 4.2%, Depreciation 1.8%, OHF 32.9%, OHDepreciation 0.5%, OHC 6.7%</t>
+          <t>CostSubmission_MF4159_2025_M07_PROD.xml: fixtures pool 14,810.610 AED placed on 9 claims by units (19 units; 779.506 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M06_PROD.xml: bucket Anaesthesia profile SWNurs 9.5%, SWDoc 74.3%, Pharmacy 16.2%</t>
+          <t>CostSubmission_MF4159_2025_M07_PROD.xml: abutments pool 6,350.000 AED placed on 16 claims by units (32 units; 198.438 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M06_PROD.xml: bucket Imaging profile SWNurs 84.9%, Depreciation 15.1%</t>
+          <t>CostSubmission_MF4159_2025_M07_PROD.xml: bone_graft pool 5,800.000 AED placed on 8 claims by units (35 units; 165.714 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t xml:space="preserve">CostSubmission_MF4159_2025_M06_PROD.xml: bucket Laboratory profile </t>
+          <t>CostSubmission_MF4159_2025_M07_PROD.xml: lab: claim 1719MF4159-6bb02a share 223.163 capped at its Dental amount 130.282</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M07_PROD.xml: claim totals -0.020 AED vs ledger absorbed by claim 2066MF4159-ff09af</t>
+          <t>CostSubmission_MF4159_2025_M07_PROD.xml: lab: claim 1936MF4159-00e706 share 148.776 capped at its Dental amount 86.855</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M07_PROD.xml: Prostheses pools fixtures 14,810.61, abutments 6,350.00, bone_graft 5,800.00, lab 19,563.99; coded claims in activity: 122</t>
+          <t>CostSubmission_MF4159_2025_M07_PROD.xml: lab: claim 2158MF4159-35df2b share 74.388 capped at its Dental amount 43.428</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M07_PROD.xml: fixtures pool 14,810.610 AED placed on 9 claims by units (19 units; 779.506 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M07_PROD.xml: lab pool 19,563.990 AED placed on 122 claims by units (263 units; 74.388 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M07_PROD.xml: abutments pool 6,350.000 AED placed on 16 claims by units (32 units; 198.438 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M07_PROD.xml: dental technicians: claim 1719MF4159-6bb02a share 71.804 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M07_PROD.xml: bone_graft pool 5,800.000 AED placed on 8 claims by units (35 units; 165.714 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M07_PROD.xml: dental technicians: claim 1936MF4159-00e706 share 47.869 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M07_PROD.xml: lab: claim 1719MF4159-6bb02a share 223.163 capped at its Dental amount 130.282</t>
+          <t>CostSubmission_MF4159_2025_M07_PROD.xml: dental technicians: claim 2158MF4159-35df2b share 23.934 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M07_PROD.xml: lab: claim 1936MF4159-00e706 share 148.776 capped at its Dental amount 86.855</t>
+          <t>CostSubmission_MF4159_2025_M07_PROD.xml: dental technicians pool 6,294.796 AED placed on 119 claims by units (263 units; 23.935 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M07_PROD.xml: lab: claim 2158MF4159-35df2b share 74.388 capped at its Dental amount 43.428</t>
+          <t>CostSubmission_MF4159_2025_M07_PROD.xml: fils residuals {SWNurs:+56, SWDoc:-63, SWAllied:+71, Pharmacy:+9, MS:-61, Depreciation:-54, OHF:+39, OHDepreciation:-29, OHC:+32} absorbed by claim index 362</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M07_PROD.xml: lab pool 19,563.990 AED placed on 122 claims by units (263 units; 74.388 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M07_PROD.xml: bucket Prosthesis profile SWNurs 5.8%, SWDoc 33.0%, SWAllied 10.0%, Prostheses 49.5%, MS 1.7%</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M07_PROD.xml: dental technicians: claim 1719MF4159-6bb02a share 71.804 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M07_PROD.xml: bucket Dental profile SWNurs 9.5%, SWDoc 33.9%, SWAllied 2.6%, Prostheses 1.3%, MS 6.0%, Depreciation 2.6%, OHF 36.5%, OHDepreciation 0.7%, OHC 6.8%</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M07_PROD.xml: dental technicians: claim 1936MF4159-00e706 share 47.869 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M07_PROD.xml: bucket Imaging profile SWNurs 9.5%, SWDoc 36.2%, SWAllied 5.2%, Prostheses 10.2%, MS 5.7%, Depreciation 2.3%, OHF 30.8%</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M07_PROD.xml: dental technicians: claim 2158MF4159-35df2b share 23.934 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M07_PROD.xml: bucket Anaesthesia profile SWNurs 13.5%, SWDoc 51.4%, Pharmacy 9.3%, Prostheses 14.4%, MS 8.1%, Depreciation 3.3%</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M07_PROD.xml: dental technicians pool 6,294.796 AED placed on 119 claims by units (263 units; 23.935 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: claim totals -0.040 AED vs ledger absorbed by claim 1749MF4159-288273</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M07_PROD.xml: fils residuals {SWNurs:+56, SWDoc:-63, SWAllied:+71, Pharmacy:+9, MS:-61, Depreciation:-54, OHF:+39, OHDepreciation:-29, OHC:+32} absorbed by claim index 362</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: Prostheses pools fixtures 24,948.24, bone_graft 4,150.00, abutments 4,900.00, lab 35,990.74; coded claims in activity: 128</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M07_PROD.xml: bucket Prosthesis profile SWAllied 11.9%, Prostheses 88.1%</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: fixtures pool 24,948.240 AED placed on 11 claims by units (34 units; 733.772 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M07_PROD.xml: bucket Dental profile SWNurs 9.8%, SWDoc 38.6%, SWAllied 2.8%, MS 6.2%, Depreciation 2.4%, OHF 33.5%, OHDepreciation 0.6%, OHC 6.0%</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: bone_graft pool 4,150.000 AED placed on 8 claims by units (45 units; 92.222 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M07_PROD.xml: bucket Anaesthesia profile SWNurs 8.3%, SWDoc 63.0%, Pharmacy 28.7%</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: abutments pool 4,900.000 AED placed on 24 claims by units (52 units; 94.231 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M07_PROD.xml: bucket Imaging profile SWNurs 80.5%, Depreciation 19.5%</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: lab: claim 2024MF4159-87c40f share 92.521 capped at its Dental amount 27.225</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t xml:space="preserve">CostSubmission_MF4159_2025_M07_PROD.xml: bucket Laboratory profile </t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: lab pool 35,990.740 AED placed on 128 claims by units (389 units; 92.521 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: claim totals -0.040 AED vs ledger absorbed by claim 1749MF4159-288273</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: dental technicians: claim 2024MF4159-87c40f share 32.893 capped at its Dental amount 0.000</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: Prostheses pools fixtures 24,948.24, bone_graft 4,150.00, abutments 4,900.00, lab 35,990.74; coded claims in activity: 128</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: dental technicians: claim 2145MF4159-7f25c0 share 32.892 capped at its Dental amount 22.873</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: fixtures pool 24,948.240 AED placed on 11 claims by units (34 units; 733.772 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: dental technicians: claim 2179MF4159-92f1be share 65.785 capped at its Dental amount 45.746</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: bone_graft pool 4,150.000 AED placed on 8 claims by units (45 units; 92.222 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: dental technicians: claim 1789MF4159-5c32d1 share 32.892 capped at its Dental amount 22.873</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: abutments pool 4,900.000 AED placed on 24 claims by units (52 units; 94.231 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: dental technicians: claim 1745MF4159-7deac0 share 98.677 capped at its Dental amount 68.619</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: lab: claim 2024MF4159-87c40f share 92.521 capped at its Dental amount 27.225</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: dental technicians: claim 389MF4159-ea32e5 share 32.892 capped at its Dental amount 22.873</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: lab pool 35,990.740 AED placed on 128 claims by units (389 units; 92.521 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: dental technicians: claim 391MF4159-5cbd8c share 32.892 capped at its Dental amount 22.874</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: dental technicians: claim 2024MF4159-87c40f share 32.893 capped at its Dental amount 0.000</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: dental technicians pool 12,795.132 AED placed on 127 claims by units (389 units; 32.892 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: dental technicians: claim 2145MF4159-7f25c0 share 32.892 capped at its Dental amount 22.873</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: fils residuals {SWNurs:-84, SWDoc:-14, SWAllied:+57, Pharmacy:+44, MS:+11, Depreciation:+16, OHF:-17, OHDepreciation:+40, OHC:-53} absorbed by claim index 157</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: dental technicians: claim 2179MF4159-92f1be share 65.785 capped at its Dental amount 45.746</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: bucket Prosthesis profile SWNurs 4.8%, SWDoc 23.5%, SWAllied 14.0%, Prostheses 56.2%, MS 1.5%</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: dental technicians: claim 1789MF4159-5c32d1 share 32.892 capped at its Dental amount 22.873</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: bucket Dental profile SWNurs 9.9%, SWDoc 30.3%, SWAllied 2.4%, Prostheses 1.8%, MS 6.7%, Depreciation 2.5%, OHF 38.7%, OHDepreciation 0.7%, OHC 7.1%</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: dental technicians: claim 1745MF4159-7deac0 share 98.677 capped at its Dental amount 68.619</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: bucket Imaging profile SWNurs 9.6%, SWDoc 31.5%, SWAllied 4.6%, Prostheses 14.2%, MS 6.1%, Depreciation 2.1%, OHF 31.8%</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: dental technicians: claim 389MF4159-ea32e5 share 32.892 capped at its Dental amount 22.873</t>
+          <t>CostSubmission_MF4159_2025_M08_PROD.xml: bucket Anaesthesia profile SWNurs 13.9%, SWDoc 45.6%, Pharmacy 8.0%, Prostheses 20.5%, MS 8.9%, Depreciation 3.1%</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: dental technicians: claim 391MF4159-5cbd8c share 32.892 capped at its Dental amount 22.874</t>
+          <t>CostSubmission_MF4159_2025_M09_PROD.xml: claim totals -0.038 AED vs ledger absorbed by claim 1478MF4159-4ccb54</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: dental technicians pool 12,795.132 AED placed on 127 claims by units (389 units; 32.892 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M09_PROD.xml: Prostheses pools abutments 2,500.00, fixtures 29,426.15, bone_graft 9,400.00, lab 16,276.17; coded claims in activity: 110</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: fils residuals {SWNurs:-84, SWDoc:-14, SWAllied:+57, Pharmacy:+44, MS:+11, Depreciation:+16, OHF:-17, OHDepreciation:+40, OHC:-53} absorbed by claim index 157</t>
+          <t>CostSubmission_MF4159_2025_M09_PROD.xml: abutments pool 2,500.000 AED placed on 21 claims by units (42 units; 59.524 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: bucket Prosthesis profile SWAllied 15.5%, Prostheses 84.5%</t>
+          <t>CostSubmission_MF4159_2025_M09_PROD.xml: fixtures pool 29,426.150 AED placed on 13 claims by units (31 units; 949.231 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: bucket Dental profile SWNurs 10.3%, SWDoc 35.0%, SWAllied 2.6%, MS 6.9%, Depreciation 2.3%, OHF 36.0%, OHDepreciation 0.6%, OHC 6.3%</t>
+          <t>CostSubmission_MF4159_2025_M09_PROD.xml: bone_graft pool 9,400.000 AED placed on 15 claims by units (67 units; 140.299 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: bucket Anaesthesia profile SWNurs 9.6%, SWDoc 62.9%, Pharmacy 27.4%</t>
+          <t>CostSubmission_MF4159_2025_M09_PROD.xml: lab pool 16,276.170 AED placed on 110 claims by units (327 units; 49.774 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M08_PROD.xml: bucket Imaging profile SWNurs 81.8%, Depreciation 18.2%</t>
+          <t>CostSubmission_MF4159_2025_M09_PROD.xml: dental technicians pool 10,676.482 AED placed on 110 claims by units (327 units; 32.650 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t xml:space="preserve">CostSubmission_MF4159_2025_M08_PROD.xml: bucket Laboratory profile </t>
+          <t>CostSubmission_MF4159_2025_M09_PROD.xml: fils residuals {SWNurs:+9, SWDoc:-16, SWAllied:+25, Pharmacy:-3, MS:+13, Depreciation:+39, OHF:-39, OHDepreciation:-50, OHC:+22} absorbed by claim index 18</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M09_PROD.xml: claim totals -0.038 AED vs ledger absorbed by claim 1478MF4159-4ccb54</t>
+          <t>CostSubmission_MF4159_2025_M09_PROD.xml: bucket Prosthesis profile SWNurs 3.5%, SWDoc 29.3%, SWAllied 13.4%, Prostheses 52.3%, MS 1.4%</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M09_PROD.xml: Prostheses pools abutments 2,500.00, fixtures 29,426.15, bone_graft 9,400.00, lab 16,276.17; coded claims in activity: 110</t>
+          <t>CostSubmission_MF4159_2025_M09_PROD.xml: bucket Dental profile SWNurs 6.5%, SWDoc 33.9%, SWAllied 2.4%, Prostheses 1.5%, MS 5.6%, Depreciation 2.5%, OHF 39.5%, OHDepreciation 0.7%, OHC 7.4%</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M09_PROD.xml: abutments pool 2,500.000 AED placed on 21 claims by units (42 units; 59.524 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M09_PROD.xml: bucket Imaging profile SWNurs 6.5%, SWDoc 36.1%, SWAllied 4.8%, Prostheses 12.1%, MS 5.3%, Depreciation 2.2%, OHF 33.1%</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M09_PROD.xml: fixtures pool 29,426.150 AED placed on 13 claims by units (31 units; 949.231 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M09_PROD.xml: bucket Anaesthesia profile SWNurs 9.1%, SWDoc 50.4%, Pharmacy 13.1%, Prostheses 16.9%, MS 7.4%, Depreciation 3.1%</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M09_PROD.xml: bone_graft pool 9,400.000 AED placed on 15 claims by units (67 units; 140.299 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M10_PROD.xml: claim totals -0.084 AED vs ledger absorbed by claim 2140MF4159-5323ad</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M09_PROD.xml: lab pool 16,276.170 AED placed on 110 claims by units (327 units; 49.774 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M10_PROD.xml: Prostheses pools abutments 3,755.00, fixtures 18,497.17, bone_graft 10,880.00, lab 16,393.19; coded claims in activity: 123</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M09_PROD.xml: dental technicians pool 10,676.482 AED placed on 110 claims by units (327 units; 32.650 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M10_PROD.xml: abutments pool 3,755.000 AED placed on 22 claims by units (36 units; 104.306 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M09_PROD.xml: fils residuals {SWNurs:+9, SWDoc:-16, SWAllied:+25, Pharmacy:-3, MS:+13, Depreciation:+39, OHF:-39, OHDepreciation:-50, OHC:+22} absorbed by claim index 18</t>
+          <t>CostSubmission_MF4159_2025_M10_PROD.xml: fixtures pool 18,497.170 AED placed on 13 claims by units (29 units; 637.833 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M09_PROD.xml: bucket Prosthesis profile SWAllied 15.6%, Prostheses 84.4%</t>
+          <t>CostSubmission_MF4159_2025_M10_PROD.xml: bone_graft pool 10,880.000 AED placed on 11 claims by units (50 units; 217.600 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M09_PROD.xml: bucket Dental profile SWNurs 6.8%, SWDoc 38.9%, SWAllied 2.6%, MS 5.8%, Depreciation 2.3%, OHF 36.5%, OHDepreciation 0.6%, OHC 6.5%</t>
+          <t>CostSubmission_MF4159_2025_M10_PROD.xml: lab pool 16,393.190 AED placed on 123 claims by units (276 units; 59.396 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M09_PROD.xml: bucket Anaesthesia profile SWNurs 5.2%, SWDoc 57.4%, Pharmacy 37.4%</t>
+          <t>CostSubmission_MF4159_2025_M10_PROD.xml: dental technicians pool 7,091.542 AED placed on 123 claims by units (276 units; 25.694 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M09_PROD.xml: bucket Imaging profile SWNurs 74.6%, Depreciation 25.4%</t>
+          <t>CostSubmission_MF4159_2025_M10_PROD.xml: fils residuals {SWNurs:+42, SWDoc:+4, SWAllied:-6, Pharmacy:-33, MS:+49, GS:-1, Depreciation:-25, OHF:+24, OHDepreciation:-43, OHC:-11} absorbed by claim index 492</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t xml:space="preserve">CostSubmission_MF4159_2025_M09_PROD.xml: bucket Laboratory profile </t>
+          <t>CostSubmission_MF4159_2025_M10_PROD.xml: bucket Prosthesis profile SWNurs 4.8%, SWDoc 38.3%, SWAllied 9.5%, Prostheses 45.9%, MS 1.4%</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M10_PROD.xml: claim totals -0.084 AED vs ledger absorbed by claim 2140MF4159-5323ad</t>
+          <t>CostSubmission_MF4159_2025_M10_PROD.xml: bucket Dental profile SWNurs 8.0%, SWDoc 39.7%, SWAllied 2.1%, Prostheses 1.2%, MS 5.1%, GS 0.3%, Depreciation 2.3%, OHF 34.5%, OHDepreciation 0.6%, OHC 6.1%</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M10_PROD.xml: Prostheses pools abutments 3,755.00, fixtures 18,497.17, bone_graft 10,880.00, lab 16,393.19; coded claims in activity: 123</t>
+          <t>CostSubmission_MF4159_2025_M10_PROD.xml: bucket Imaging profile SWNurs 8.0%, SWDoc 42.3%, SWAllied 4.2%, Prostheses 9.5%, MS 4.8%, Depreciation 2.0%, OHF 29.1%</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M10_PROD.xml: abutments pool 3,755.000 AED placed on 22 claims by units (36 units; 104.306 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M10_PROD.xml: bucket Anaesthesia profile SWNurs 11.2%, SWDoc 59.6%, Pharmacy 6.2%, Prostheses 13.4%, MS 6.8%, Depreciation 2.9%</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M10_PROD.xml: fixtures pool 18,497.170 AED placed on 13 claims by units (29 units; 637.833 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M11_PROD.xml: claim totals -0.041 AED vs ledger absorbed by claim 1738MF4159-0b278e</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M10_PROD.xml: bone_graft pool 10,880.000 AED placed on 11 claims by units (50 units; 217.600 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M11_PROD.xml: Prostheses pools abutments 2,745.00, fixtures 9,022.73, bone_graft 6,225.00, lab 35,933.97; coded claims in activity: 107</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M10_PROD.xml: lab pool 16,393.190 AED placed on 123 claims by units (276 units; 59.396 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M11_PROD.xml: abutments pool 2,745.000 AED placed on 20 claims by units (40 units; 68.625 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M10_PROD.xml: dental technicians pool 7,091.542 AED placed on 123 claims by units (276 units; 25.694 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M11_PROD.xml: fixtures pool 9,022.730 AED placed on 10 claims by units (17 units; 530.749 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M10_PROD.xml: fils residuals {SWNurs:+42, SWDoc:+4, SWAllied:-6, Pharmacy:-33, MS:+49, GS:-1, Depreciation:-25, OHF:+24, OHDepreciation:-43, OHC:-11} absorbed by claim index 492</t>
+          <t>CostSubmission_MF4159_2025_M11_PROD.xml: bone_graft pool 6,225.000 AED placed on 13 claims by units (30 units; 207.500 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M10_PROD.xml: bucket Prosthesis profile SWAllied 12.5%, Prostheses 87.5%</t>
+          <t>CostSubmission_MF4159_2025_M11_PROD.xml: lab pool 35,933.970 AED placed on 107 claims by units (249 units; 144.313 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M10_PROD.xml: bucket Dental profile SWNurs 8.2%, SWDoc 44.8%, SWAllied 2.3%, MS 5.2%, GS 0.3%, Depreciation 2.1%, OHF 31.4%, OHDepreciation 0.5%, OHC 5.3%</t>
+          <t>CostSubmission_MF4159_2025_M11_PROD.xml: dental technicians pool 10,339.683 AED placed on 107 claims by units (249 units; 41.525 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M10_PROD.xml: bucket Anaesthesia profile SWNurs 7.0%, SWDoc 73.8%, Pharmacy 19.2%</t>
+          <t>CostSubmission_MF4159_2025_M11_PROD.xml: fils residuals {SWNurs:+28, SWDoc:+18, SWAllied:-8, Pharmacy:+23, MS:-10, Depreciation:-92, OHF:+46, OHDepreciation:+49, OHC:-54} absorbed by claim index 81</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M10_PROD.xml: bucket Imaging profile SWNurs 79.7%, Depreciation 20.3%</t>
+          <t>CostSubmission_MF4159_2025_M11_PROD.xml: bucket Prosthesis profile SWNurs 4.7%, SWDoc 28.5%, SWAllied 13.6%, Prostheses 51.7%, MS 1.5%</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t xml:space="preserve">CostSubmission_MF4159_2025_M10_PROD.xml: bucket Laboratory profile </t>
+          <t>CostSubmission_MF4159_2025_M11_PROD.xml: bucket Dental profile SWNurs 8.4%, SWDoc 32.0%, SWAllied 2.2%, Prostheses 1.5%, MS 5.7%, Depreciation 2.6%, OHF 40.3%, OHDepreciation 0.7%, OHC 6.7%</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M11_PROD.xml: claim totals -0.041 AED vs ledger absorbed by claim 1738MF4159-0b278e</t>
+          <t>CostSubmission_MF4159_2025_M11_PROD.xml: bucket Imaging profile SWNurs 8.4%, SWDoc 34.2%, SWAllied 4.3%, Prostheses 11.6%, MS 5.4%, Depreciation 2.3%, OHF 33.9%</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M11_PROD.xml: Prostheses pools abutments 2,745.00, fixtures 9,022.73, bone_graft 6,225.00, lab 35,933.97; coded claims in activity: 107</t>
+          <t>CostSubmission_MF4159_2025_M11_PROD.xml: bucket Anaesthesia profile SWNurs 12.5%, SWDoc 51.0%, Pharmacy 7.7%, Prostheses 17.3%, MS 8.1%, Depreciation 3.4%</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M11_PROD.xml: abutments pool 2,745.000 AED placed on 20 claims by units (40 units; 68.625 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: claim totals +0.061 AED vs ledger absorbed by claim 2043MF4159-174974</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M11_PROD.xml: fixtures pool 9,022.730 AED placed on 10 claims by units (17 units; 530.749 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: Prostheses pools abutments 1,850.00, fixtures 16,598.48, bone_graft 9,450.00, lab 41,042.50; coded claims in activity: 115</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M11_PROD.xml: bone_graft pool 6,225.000 AED placed on 13 claims by units (30 units; 207.500 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: abutments pool 1,850.000 AED placed on 20 claims by units (37 units; 50.000 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M11_PROD.xml: lab pool 35,933.970 AED placed on 107 claims by units (249 units; 144.313 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: fixtures pool 16,598.480 AED placed on 10 claims by units (15 units; 1,106.565 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M11_PROD.xml: dental technicians pool 10,339.683 AED placed on 107 claims by units (249 units; 41.525 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: bone_graft pool 9,450.000 AED placed on 8 claims by units (26 units; 363.462 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M11_PROD.xml: fils residuals {SWNurs:+28, SWDoc:+18, SWAllied:-8, Pharmacy:+23, MS:-10, Depreciation:-92, OHF:+46, OHDepreciation:+49, OHC:-54} absorbed by claim index 81</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: lab pool 41,042.500 AED placed on 115 claims by units (259 units; 158.465 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M11_PROD.xml: bucket Prosthesis profile SWAllied 16.1%, Prostheses 83.9%</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians: claim 2073MF4159-5b1531 share 75.348 capped at its Dental amount 56.779</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M11_PROD.xml: bucket Dental profile SWNurs 8.7%, SWDoc 36.8%, SWAllied 2.4%, MS 5.9%, Depreciation 2.4%, OHF 37.2%, OHDepreciation 0.6%, OHC 5.9%</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians: claim 2095MF4159-4d3bdb share 75.348 capped at its Dental amount 56.779</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M11_PROD.xml: bucket Anaesthesia profile SWNurs 8.1%, SWDoc 66.6%, Pharmacy 25.2%</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians: claim 2123MF4159-237d2d share 75.348 capped at its Dental amount 56.779</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M11_PROD.xml: bucket Imaging profile SWNurs 78.6%, Depreciation 21.4%</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians: claim 2128MF4159-e95eeb share 75.348 capped at its Dental amount 56.779</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t xml:space="preserve">CostSubmission_MF4159_2025_M11_PROD.xml: bucket Laboratory profile </t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians: claim 2135MF4159-8747a5 share 150.696 capped at its Dental amount 113.557</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: claim totals +0.061 AED vs ledger absorbed by claim 2043MF4159-174974</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians: claim 2175MF4159-57b801 share 75.348 capped at its Dental amount 56.779</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: Prostheses pools abutments 1,850.00, fixtures 16,598.48, bone_graft 9,450.00, lab 41,042.50; coded claims in activity: 115</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians: claim 2197MF4159-9b3fae share 75.348 capped at its Dental amount 56.779</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: abutments pool 1,850.000 AED placed on 20 claims by units (37 units; 50.000 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians: claim 2212MF4159-1be1ce share 904.174 capped at its Dental amount 788.968</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: fixtures pool 16,598.480 AED placed on 10 claims by units (15 units; 1,106.565 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians: claim 2245MF4159-c3ee38 share 75.348 capped at its Dental amount 56.779</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: bone_graft pool 9,450.000 AED placed on 8 claims by units (26 units; 363.462 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians: claim 2249MF4159-58a8a6 share 75.348 capped at its Dental amount 56.779</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: lab pool 41,042.500 AED placed on 115 claims by units (259 units; 158.465 AED per unit)</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians: claim 2264MF4159-5a1d74 share 150.695 capped at its Dental amount 113.557</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians: claim 2073MF4159-5b1531 share 75.348 capped at its Dental amount 56.779</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians pool 19,515.095 AED placed on 115 claims by units (259 units; 75.348 AED per unit)</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians: claim 2095MF4159-4d3bdb share 75.348 capped at its Dental amount 56.779</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: fils residuals {SWNurs:+34, SWDoc:+10, SWAllied:+16, Pharmacy:+51, MS:-66, GS:+52, Depreciation:-79, OHF:-1, OHDepreciation:+41, OHC:-58} absorbed by claim index 134</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians: claim 2123MF4159-237d2d share 75.348 capped at its Dental amount 56.779</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: bucket Prosthesis profile SWNurs 3.9%, SWDoc 31.2%, SWAllied 17.5%, Prostheses 46.4%, MS 1.0%</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians: claim 2128MF4159-e95eeb share 75.348 capped at its Dental amount 56.779</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: bucket Dental profile SWNurs 8.2%, SWDoc 40.7%, SWAllied 2.2%, Prostheses 1.5%, MS 4.4%, GS 0.0%, Depreciation 2.1%, OHF 34.8%, OHDepreciation 0.6%, OHC 5.5%</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians: claim 2135MF4159-8747a5 share 150.696 capped at its Dental amount 113.557</t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: bucket Imaging profile SWNurs 7.9%, SWDoc 42.0%, SWAllied 4.3%, Prostheses 11.7%, MS 4.0%, Depreciation 1.8%, OHF 28.3%</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians: claim 2175MF4159-57b801 share 75.348 capped at its Dental amount 56.779</t>
-        </is>
-      </c>
-    </row>
-    <row r="251">
-      <c r="A251" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians: claim 2197MF4159-9b3fae share 75.348 capped at its Dental amount 56.779</t>
-        </is>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians: claim 2212MF4159-1be1ce share 904.174 capped at its Dental amount 788.968</t>
-        </is>
-      </c>
-    </row>
-    <row r="253">
-      <c r="A253" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians: claim 2245MF4159-c3ee38 share 75.348 capped at its Dental amount 56.779</t>
-        </is>
-      </c>
-    </row>
-    <row r="254">
-      <c r="A254" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians: claim 2249MF4159-58a8a6 share 75.348 capped at its Dental amount 56.779</t>
-        </is>
-      </c>
-    </row>
-    <row r="255">
-      <c r="A255" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians: claim 2264MF4159-5a1d74 share 150.695 capped at its Dental amount 113.557</t>
-        </is>
-      </c>
-    </row>
-    <row r="256">
-      <c r="A256" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: dental technicians pool 19,515.095 AED placed on 115 claims by units (259 units; 75.348 AED per unit)</t>
-        </is>
-      </c>
-    </row>
-    <row r="257">
-      <c r="A257" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: fils residuals {SWNurs:+34, SWDoc:+10, SWAllied:+16, Pharmacy:+51, MS:-66, GS:+52, Depreciation:-79, OHF:-1, OHDepreciation:+41, OHC:-58} absorbed by claim index 134</t>
-        </is>
-      </c>
-    </row>
-    <row r="258">
-      <c r="A258" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: bucket Prosthesis profile SWAllied 22.1%, Prostheses 77.9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="259">
-      <c r="A259" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: bucket Dental profile SWNurs 8.4%, SWDoc 46.0%, SWAllied 2.4%, MS 4.4%, GS 0.0%, Depreciation 1.9%, OHF 31.6%, OHDepreciation 0.5%, OHC 4.8%</t>
-        </is>
-      </c>
-    </row>
-    <row r="260">
-      <c r="A260" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: bucket Anaesthesia profile SWNurs 7.5%, SWDoc 79.8%, Pharmacy 12.7%</t>
-        </is>
-      </c>
-    </row>
-    <row r="261">
-      <c r="A261" t="inlineStr">
-        <is>
-          <t>CostSubmission_MF4159_2025_M12_PROD.xml: bucket Imaging profile SWNurs 81.5%, Depreciation 18.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="262">
-      <c r="A262" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CostSubmission_MF4159_2025_M12_PROD.xml: bucket Laboratory profile </t>
+          <t>CostSubmission_MF4159_2025_M12_PROD.xml: bucket Anaesthesia profile SWNurs 11.3%, SWDoc 59.9%, Pharmacy 3.8%, Prostheses 16.7%, MS 5.7%, Depreciation 2.6%</t>
         </is>
       </c>
     </row>

</xml_diff>